<commit_message>
Support two-judge class imports
</commit_message>
<xml_diff>
--- a/public/hcqha-class-list-template.xlsx
+++ b/public/hcqha-class-list-template.xlsx
@@ -397,12 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C197"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="48.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D197"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,7 +407,10 @@
         <v>Class Name</v>
       </c>
       <c r="C1" t="str">
-        <v>Judge</v>
+        <v>Judge 1</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Judge 2</v>
       </c>
     </row>
     <row r="2">
@@ -425,6 +423,9 @@
       <c r="C2" t="str">
         <v/>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -436,6 +437,9 @@
       <c r="C3" t="str">
         <v/>
       </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -447,6 +451,9 @@
       <c r="C4" t="str">
         <v/>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -458,6 +465,9 @@
       <c r="C5" t="str">
         <v/>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -469,6 +479,9 @@
       <c r="C6" t="str">
         <v/>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -480,6 +493,9 @@
       <c r="C7" t="str">
         <v/>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -491,6 +507,9 @@
       <c r="C8" t="str">
         <v/>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -502,6 +521,9 @@
       <c r="C9" t="str">
         <v/>
       </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -513,6 +535,9 @@
       <c r="C10" t="str">
         <v/>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -524,6 +549,9 @@
       <c r="C11" t="str">
         <v/>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -535,6 +563,9 @@
       <c r="C12" t="str">
         <v/>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -546,6 +577,9 @@
       <c r="C13" t="str">
         <v/>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -557,6 +591,9 @@
       <c r="C14" t="str">
         <v/>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -568,6 +605,9 @@
       <c r="C15" t="str">
         <v/>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -579,6 +619,9 @@
       <c r="C16" t="str">
         <v/>
       </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -590,6 +633,9 @@
       <c r="C17" t="str">
         <v/>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -601,6 +647,9 @@
       <c r="C18" t="str">
         <v/>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -612,6 +661,9 @@
       <c r="C19" t="str">
         <v/>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -623,6 +675,9 @@
       <c r="C20" t="str">
         <v/>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -634,6 +689,9 @@
       <c r="C21" t="str">
         <v/>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -645,6 +703,9 @@
       <c r="C22" t="str">
         <v/>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -656,6 +717,9 @@
       <c r="C23" t="str">
         <v/>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -667,6 +731,9 @@
       <c r="C24" t="str">
         <v/>
       </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -678,6 +745,9 @@
       <c r="C25" t="str">
         <v/>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -689,6 +759,9 @@
       <c r="C26" t="str">
         <v/>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -700,6 +773,9 @@
       <c r="C27" t="str">
         <v/>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -711,6 +787,9 @@
       <c r="C28" t="str">
         <v/>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -722,6 +801,9 @@
       <c r="C29" t="str">
         <v/>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -733,6 +815,9 @@
       <c r="C30" t="str">
         <v/>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -744,6 +829,9 @@
       <c r="C31" t="str">
         <v/>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -755,6 +843,9 @@
       <c r="C32" t="str">
         <v/>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -766,6 +857,9 @@
       <c r="C33" t="str">
         <v/>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -777,6 +871,9 @@
       <c r="C34" t="str">
         <v/>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -788,6 +885,9 @@
       <c r="C35" t="str">
         <v/>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -799,6 +899,9 @@
       <c r="C36" t="str">
         <v/>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -810,6 +913,9 @@
       <c r="C37" t="str">
         <v/>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -821,6 +927,9 @@
       <c r="C38" t="str">
         <v/>
       </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -832,6 +941,9 @@
       <c r="C39" t="str">
         <v/>
       </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -843,6 +955,9 @@
       <c r="C40" t="str">
         <v/>
       </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -854,6 +969,9 @@
       <c r="C41" t="str">
         <v/>
       </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -865,6 +983,9 @@
       <c r="C42" t="str">
         <v/>
       </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -876,6 +997,9 @@
       <c r="C43" t="str">
         <v/>
       </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -887,6 +1011,9 @@
       <c r="C44" t="str">
         <v/>
       </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -898,6 +1025,9 @@
       <c r="C45" t="str">
         <v/>
       </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -909,6 +1039,9 @@
       <c r="C46" t="str">
         <v/>
       </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -920,6 +1053,9 @@
       <c r="C47" t="str">
         <v/>
       </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -931,6 +1067,9 @@
       <c r="C48" t="str">
         <v/>
       </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -942,6 +1081,9 @@
       <c r="C49" t="str">
         <v/>
       </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -953,6 +1095,9 @@
       <c r="C50" t="str">
         <v/>
       </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -964,6 +1109,9 @@
       <c r="C51" t="str">
         <v/>
       </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -975,6 +1123,9 @@
       <c r="C52" t="str">
         <v/>
       </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -986,6 +1137,9 @@
       <c r="C53" t="str">
         <v/>
       </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -997,6 +1151,9 @@
       <c r="C54" t="str">
         <v/>
       </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -1008,6 +1165,9 @@
       <c r="C55" t="str">
         <v/>
       </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -1019,6 +1179,9 @@
       <c r="C56" t="str">
         <v/>
       </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -1030,6 +1193,9 @@
       <c r="C57" t="str">
         <v/>
       </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -1041,6 +1207,9 @@
       <c r="C58" t="str">
         <v/>
       </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -1052,6 +1221,9 @@
       <c r="C59" t="str">
         <v/>
       </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -1063,6 +1235,9 @@
       <c r="C60" t="str">
         <v/>
       </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -1074,6 +1249,9 @@
       <c r="C61" t="str">
         <v/>
       </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -1085,6 +1263,9 @@
       <c r="C62" t="str">
         <v/>
       </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -1096,6 +1277,9 @@
       <c r="C63" t="str">
         <v/>
       </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -1107,6 +1291,9 @@
       <c r="C64" t="str">
         <v/>
       </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65">
@@ -1118,6 +1305,9 @@
       <c r="C65" t="str">
         <v/>
       </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66">
@@ -1129,6 +1319,9 @@
       <c r="C66" t="str">
         <v/>
       </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67">
@@ -1140,6 +1333,9 @@
       <c r="C67" t="str">
         <v/>
       </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68">
@@ -1151,6 +1347,9 @@
       <c r="C68" t="str">
         <v/>
       </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69">
@@ -1162,6 +1361,9 @@
       <c r="C69" t="str">
         <v/>
       </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70">
@@ -1173,6 +1375,9 @@
       <c r="C70" t="str">
         <v/>
       </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71">
@@ -1184,6 +1389,9 @@
       <c r="C71" t="str">
         <v/>
       </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72">
@@ -1195,6 +1403,9 @@
       <c r="C72" t="str">
         <v/>
       </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73">
@@ -1206,6 +1417,9 @@
       <c r="C73" t="str">
         <v/>
       </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74">
@@ -1217,6 +1431,9 @@
       <c r="C74" t="str">
         <v/>
       </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75">
@@ -1228,6 +1445,9 @@
       <c r="C75" t="str">
         <v/>
       </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76">
@@ -1239,6 +1459,9 @@
       <c r="C76" t="str">
         <v/>
       </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77">
@@ -1250,6 +1473,9 @@
       <c r="C77" t="str">
         <v/>
       </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78">
@@ -1261,6 +1487,9 @@
       <c r="C78" t="str">
         <v/>
       </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79">
@@ -1272,6 +1501,9 @@
       <c r="C79" t="str">
         <v/>
       </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80">
@@ -1283,6 +1515,9 @@
       <c r="C80" t="str">
         <v/>
       </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81">
@@ -1294,6 +1529,9 @@
       <c r="C81" t="str">
         <v/>
       </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82">
@@ -1305,6 +1543,9 @@
       <c r="C82" t="str">
         <v/>
       </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83">
@@ -1316,6 +1557,9 @@
       <c r="C83" t="str">
         <v/>
       </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84">
@@ -1327,6 +1571,9 @@
       <c r="C84" t="str">
         <v/>
       </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85">
@@ -1338,6 +1585,9 @@
       <c r="C85" t="str">
         <v/>
       </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86">
@@ -1349,6 +1599,9 @@
       <c r="C86" t="str">
         <v/>
       </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87">
@@ -1360,6 +1613,9 @@
       <c r="C87" t="str">
         <v/>
       </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88">
@@ -1371,6 +1627,9 @@
       <c r="C88" t="str">
         <v/>
       </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89">
@@ -1382,6 +1641,9 @@
       <c r="C89" t="str">
         <v/>
       </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90">
@@ -1393,6 +1655,9 @@
       <c r="C90" t="str">
         <v/>
       </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91">
@@ -1404,6 +1669,9 @@
       <c r="C91" t="str">
         <v/>
       </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92">
@@ -1415,6 +1683,9 @@
       <c r="C92" t="str">
         <v/>
       </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93">
@@ -1426,6 +1697,9 @@
       <c r="C93" t="str">
         <v/>
       </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94">
@@ -1437,6 +1711,9 @@
       <c r="C94" t="str">
         <v/>
       </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95">
@@ -1448,6 +1725,9 @@
       <c r="C95" t="str">
         <v/>
       </c>
+      <c r="D95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96">
@@ -1459,6 +1739,9 @@
       <c r="C96" t="str">
         <v/>
       </c>
+      <c r="D96" t="str">
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97">
@@ -1470,6 +1753,9 @@
       <c r="C97" t="str">
         <v/>
       </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98">
@@ -1481,6 +1767,9 @@
       <c r="C98" t="str">
         <v/>
       </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99">
@@ -1492,6 +1781,9 @@
       <c r="C99" t="str">
         <v/>
       </c>
+      <c r="D99" t="str">
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100">
@@ -1503,6 +1795,9 @@
       <c r="C100" t="str">
         <v/>
       </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101">
@@ -1514,6 +1809,9 @@
       <c r="C101" t="str">
         <v/>
       </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102">
@@ -1525,6 +1823,9 @@
       <c r="C102" t="str">
         <v/>
       </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103">
@@ -1536,6 +1837,9 @@
       <c r="C103" t="str">
         <v/>
       </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104">
@@ -1547,6 +1851,9 @@
       <c r="C104" t="str">
         <v/>
       </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105">
@@ -1558,6 +1865,9 @@
       <c r="C105" t="str">
         <v/>
       </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106">
@@ -1569,6 +1879,9 @@
       <c r="C106" t="str">
         <v/>
       </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107">
@@ -1580,6 +1893,9 @@
       <c r="C107" t="str">
         <v/>
       </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108">
@@ -1591,6 +1907,9 @@
       <c r="C108" t="str">
         <v/>
       </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109">
@@ -1602,6 +1921,9 @@
       <c r="C109" t="str">
         <v/>
       </c>
+      <c r="D109" t="str">
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110">
@@ -1613,6 +1935,9 @@
       <c r="C110" t="str">
         <v/>
       </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111">
@@ -1624,6 +1949,9 @@
       <c r="C111" t="str">
         <v/>
       </c>
+      <c r="D111" t="str">
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112">
@@ -1635,6 +1963,9 @@
       <c r="C112" t="str">
         <v/>
       </c>
+      <c r="D112" t="str">
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113">
@@ -1646,6 +1977,9 @@
       <c r="C113" t="str">
         <v/>
       </c>
+      <c r="D113" t="str">
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114">
@@ -1657,6 +1991,9 @@
       <c r="C114" t="str">
         <v/>
       </c>
+      <c r="D114" t="str">
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115">
@@ -1668,6 +2005,9 @@
       <c r="C115" t="str">
         <v/>
       </c>
+      <c r="D115" t="str">
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116">
@@ -1679,6 +2019,9 @@
       <c r="C116" t="str">
         <v/>
       </c>
+      <c r="D116" t="str">
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117">
@@ -1690,6 +2033,9 @@
       <c r="C117" t="str">
         <v/>
       </c>
+      <c r="D117" t="str">
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118">
@@ -1701,6 +2047,9 @@
       <c r="C118" t="str">
         <v/>
       </c>
+      <c r="D118" t="str">
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119">
@@ -1712,6 +2061,9 @@
       <c r="C119" t="str">
         <v/>
       </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120">
@@ -1723,6 +2075,9 @@
       <c r="C120" t="str">
         <v/>
       </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121">
@@ -1734,6 +2089,9 @@
       <c r="C121" t="str">
         <v/>
       </c>
+      <c r="D121" t="str">
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122">
@@ -1745,6 +2103,9 @@
       <c r="C122" t="str">
         <v/>
       </c>
+      <c r="D122" t="str">
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123">
@@ -1756,6 +2117,9 @@
       <c r="C123" t="str">
         <v/>
       </c>
+      <c r="D123" t="str">
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124">
@@ -1767,6 +2131,9 @@
       <c r="C124" t="str">
         <v/>
       </c>
+      <c r="D124" t="str">
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125">
@@ -1778,6 +2145,9 @@
       <c r="C125" t="str">
         <v/>
       </c>
+      <c r="D125" t="str">
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126">
@@ -1789,6 +2159,9 @@
       <c r="C126" t="str">
         <v/>
       </c>
+      <c r="D126" t="str">
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127">
@@ -1800,6 +2173,9 @@
       <c r="C127" t="str">
         <v/>
       </c>
+      <c r="D127" t="str">
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128">
@@ -1811,6 +2187,9 @@
       <c r="C128" t="str">
         <v/>
       </c>
+      <c r="D128" t="str">
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129">
@@ -1822,6 +2201,9 @@
       <c r="C129" t="str">
         <v/>
       </c>
+      <c r="D129" t="str">
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130">
@@ -1833,6 +2215,9 @@
       <c r="C130" t="str">
         <v/>
       </c>
+      <c r="D130" t="str">
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131">
@@ -1844,6 +2229,9 @@
       <c r="C131" t="str">
         <v/>
       </c>
+      <c r="D131" t="str">
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132">
@@ -1855,6 +2243,9 @@
       <c r="C132" t="str">
         <v/>
       </c>
+      <c r="D132" t="str">
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133">
@@ -1866,6 +2257,9 @@
       <c r="C133" t="str">
         <v/>
       </c>
+      <c r="D133" t="str">
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134">
@@ -1877,6 +2271,9 @@
       <c r="C134" t="str">
         <v/>
       </c>
+      <c r="D134" t="str">
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135">
@@ -1888,6 +2285,9 @@
       <c r="C135" t="str">
         <v/>
       </c>
+      <c r="D135" t="str">
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136">
@@ -1899,6 +2299,9 @@
       <c r="C136" t="str">
         <v/>
       </c>
+      <c r="D136" t="str">
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137">
@@ -1910,6 +2313,9 @@
       <c r="C137" t="str">
         <v/>
       </c>
+      <c r="D137" t="str">
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138">
@@ -1921,6 +2327,9 @@
       <c r="C138" t="str">
         <v/>
       </c>
+      <c r="D138" t="str">
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139">
@@ -1932,6 +2341,9 @@
       <c r="C139" t="str">
         <v/>
       </c>
+      <c r="D139" t="str">
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140">
@@ -1943,6 +2355,9 @@
       <c r="C140" t="str">
         <v/>
       </c>
+      <c r="D140" t="str">
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141">
@@ -1954,6 +2369,9 @@
       <c r="C141" t="str">
         <v/>
       </c>
+      <c r="D141" t="str">
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142">
@@ -1965,6 +2383,9 @@
       <c r="C142" t="str">
         <v/>
       </c>
+      <c r="D142" t="str">
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143">
@@ -1976,6 +2397,9 @@
       <c r="C143" t="str">
         <v/>
       </c>
+      <c r="D143" t="str">
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144">
@@ -1987,6 +2411,9 @@
       <c r="C144" t="str">
         <v/>
       </c>
+      <c r="D144" t="str">
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145">
@@ -1998,6 +2425,9 @@
       <c r="C145" t="str">
         <v/>
       </c>
+      <c r="D145" t="str">
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146">
@@ -2009,6 +2439,9 @@
       <c r="C146" t="str">
         <v/>
       </c>
+      <c r="D146" t="str">
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147">
@@ -2020,6 +2453,9 @@
       <c r="C147" t="str">
         <v/>
       </c>
+      <c r="D147" t="str">
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148">
@@ -2031,6 +2467,9 @@
       <c r="C148" t="str">
         <v/>
       </c>
+      <c r="D148" t="str">
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149">
@@ -2042,6 +2481,9 @@
       <c r="C149" t="str">
         <v/>
       </c>
+      <c r="D149" t="str">
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150">
@@ -2053,6 +2495,9 @@
       <c r="C150" t="str">
         <v/>
       </c>
+      <c r="D150" t="str">
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151">
@@ -2064,6 +2509,9 @@
       <c r="C151" t="str">
         <v/>
       </c>
+      <c r="D151" t="str">
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152">
@@ -2075,6 +2523,9 @@
       <c r="C152" t="str">
         <v/>
       </c>
+      <c r="D152" t="str">
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153">
@@ -2086,6 +2537,9 @@
       <c r="C153" t="str">
         <v/>
       </c>
+      <c r="D153" t="str">
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154">
@@ -2097,6 +2551,9 @@
       <c r="C154" t="str">
         <v/>
       </c>
+      <c r="D154" t="str">
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155">
@@ -2108,6 +2565,9 @@
       <c r="C155" t="str">
         <v/>
       </c>
+      <c r="D155" t="str">
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156">
@@ -2119,6 +2579,9 @@
       <c r="C156" t="str">
         <v/>
       </c>
+      <c r="D156" t="str">
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157">
@@ -2130,6 +2593,9 @@
       <c r="C157" t="str">
         <v/>
       </c>
+      <c r="D157" t="str">
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158">
@@ -2141,6 +2607,9 @@
       <c r="C158" t="str">
         <v/>
       </c>
+      <c r="D158" t="str">
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159">
@@ -2152,6 +2621,9 @@
       <c r="C159" t="str">
         <v/>
       </c>
+      <c r="D159" t="str">
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160">
@@ -2163,6 +2635,9 @@
       <c r="C160" t="str">
         <v/>
       </c>
+      <c r="D160" t="str">
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161">
@@ -2174,6 +2649,9 @@
       <c r="C161" t="str">
         <v/>
       </c>
+      <c r="D161" t="str">
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162">
@@ -2185,6 +2663,9 @@
       <c r="C162" t="str">
         <v/>
       </c>
+      <c r="D162" t="str">
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163">
@@ -2196,6 +2677,9 @@
       <c r="C163" t="str">
         <v/>
       </c>
+      <c r="D163" t="str">
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164">
@@ -2207,6 +2691,9 @@
       <c r="C164" t="str">
         <v/>
       </c>
+      <c r="D164" t="str">
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165">
@@ -2218,6 +2705,9 @@
       <c r="C165" t="str">
         <v/>
       </c>
+      <c r="D165" t="str">
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166">
@@ -2229,6 +2719,9 @@
       <c r="C166" t="str">
         <v/>
       </c>
+      <c r="D166" t="str">
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167">
@@ -2240,6 +2733,9 @@
       <c r="C167" t="str">
         <v/>
       </c>
+      <c r="D167" t="str">
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168">
@@ -2251,6 +2747,9 @@
       <c r="C168" t="str">
         <v/>
       </c>
+      <c r="D168" t="str">
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169">
@@ -2262,6 +2761,9 @@
       <c r="C169" t="str">
         <v/>
       </c>
+      <c r="D169" t="str">
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170">
@@ -2273,6 +2775,9 @@
       <c r="C170" t="str">
         <v/>
       </c>
+      <c r="D170" t="str">
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171">
@@ -2284,6 +2789,9 @@
       <c r="C171" t="str">
         <v/>
       </c>
+      <c r="D171" t="str">
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172">
@@ -2295,6 +2803,9 @@
       <c r="C172" t="str">
         <v/>
       </c>
+      <c r="D172" t="str">
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173">
@@ -2306,6 +2817,9 @@
       <c r="C173" t="str">
         <v/>
       </c>
+      <c r="D173" t="str">
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174">
@@ -2317,6 +2831,9 @@
       <c r="C174" t="str">
         <v/>
       </c>
+      <c r="D174" t="str">
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175">
@@ -2328,6 +2845,9 @@
       <c r="C175" t="str">
         <v/>
       </c>
+      <c r="D175" t="str">
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176">
@@ -2339,6 +2859,9 @@
       <c r="C176" t="str">
         <v/>
       </c>
+      <c r="D176" t="str">
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177">
@@ -2350,6 +2873,9 @@
       <c r="C177" t="str">
         <v/>
       </c>
+      <c r="D177" t="str">
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178">
@@ -2361,6 +2887,9 @@
       <c r="C178" t="str">
         <v/>
       </c>
+      <c r="D178" t="str">
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179">
@@ -2372,6 +2901,9 @@
       <c r="C179" t="str">
         <v/>
       </c>
+      <c r="D179" t="str">
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180">
@@ -2383,6 +2915,9 @@
       <c r="C180" t="str">
         <v/>
       </c>
+      <c r="D180" t="str">
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181">
@@ -2394,6 +2929,9 @@
       <c r="C181" t="str">
         <v/>
       </c>
+      <c r="D181" t="str">
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182">
@@ -2405,6 +2943,9 @@
       <c r="C182" t="str">
         <v/>
       </c>
+      <c r="D182" t="str">
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183">
@@ -2416,6 +2957,9 @@
       <c r="C183" t="str">
         <v/>
       </c>
+      <c r="D183" t="str">
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184">
@@ -2427,6 +2971,9 @@
       <c r="C184" t="str">
         <v/>
       </c>
+      <c r="D184" t="str">
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185">
@@ -2438,6 +2985,9 @@
       <c r="C185" t="str">
         <v/>
       </c>
+      <c r="D185" t="str">
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186">
@@ -2449,6 +2999,9 @@
       <c r="C186" t="str">
         <v/>
       </c>
+      <c r="D186" t="str">
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187">
@@ -2460,6 +3013,9 @@
       <c r="C187" t="str">
         <v/>
       </c>
+      <c r="D187" t="str">
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="A188">
@@ -2471,6 +3027,9 @@
       <c r="C188" t="str">
         <v/>
       </c>
+      <c r="D188" t="str">
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="A189">
@@ -2482,6 +3041,9 @@
       <c r="C189" t="str">
         <v/>
       </c>
+      <c r="D189" t="str">
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="A190">
@@ -2493,6 +3055,9 @@
       <c r="C190" t="str">
         <v/>
       </c>
+      <c r="D190" t="str">
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="A191">
@@ -2504,6 +3069,9 @@
       <c r="C191" t="str">
         <v/>
       </c>
+      <c r="D191" t="str">
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192">
@@ -2515,6 +3083,9 @@
       <c r="C192" t="str">
         <v/>
       </c>
+      <c r="D192" t="str">
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193">
@@ -2526,6 +3097,9 @@
       <c r="C193" t="str">
         <v/>
       </c>
+      <c r="D193" t="str">
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194">
@@ -2537,6 +3111,9 @@
       <c r="C194" t="str">
         <v/>
       </c>
+      <c r="D194" t="str">
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195">
@@ -2548,6 +3125,9 @@
       <c r="C195" t="str">
         <v/>
       </c>
+      <c r="D195" t="str">
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196">
@@ -2559,6 +3139,9 @@
       <c r="C196" t="str">
         <v/>
       </c>
+      <c r="D196" t="str">
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197">
@@ -2570,10 +3153,13 @@
       <c r="C197" t="str">
         <v/>
       </c>
+      <c r="D197" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C197"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D197"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add class program categories
</commit_message>
<xml_diff>
--- a/public/hcqha-class-list-template.xlsx
+++ b/public/hcqha-class-list-template.xlsx
@@ -397,2769 +397,3360 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D197"/>
+  <dimension ref="A1:E197"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="B1" t="str">
         <v>Class #</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Class Name</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Judge 1</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Judge 2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B2">
         <v>1</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>QH Colt 1 year &amp; under</v>
       </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
       <c r="D2" t="str">
         <v/>
       </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B3">
         <v>2</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>QH Colt 2 &amp; 3 years</v>
       </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
       <c r="D3" t="str">
         <v/>
       </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B4">
         <v>3</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
         <v>QH Stallion 4 yrs &amp; over</v>
       </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
       <c r="D4" t="str">
         <v/>
       </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
-      <c r="A5">
+      <c r="A5" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B5">
         <v>4</v>
       </c>
-      <c r="B5" t="str">
+      <c r="C5" t="str">
         <v>QH Champ &amp; Reserve Colt/Stallion</v>
       </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
       <c r="D5" t="str">
         <v/>
       </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B6">
         <v>5</v>
       </c>
-      <c r="B6" t="str">
+      <c r="C6" t="str">
         <v>QH Amateur Owner Colt 3 yrs &amp; under</v>
       </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
       <c r="D6" t="str">
         <v/>
       </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="A7">
+      <c r="A7" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B7">
         <v>6</v>
       </c>
-      <c r="B7" t="str">
+      <c r="C7" t="str">
         <v>QH Amateur Owner Stallion 4 yrs &amp; over</v>
       </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
       <c r="D7" t="str">
         <v/>
       </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8">
+      <c r="A8" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B8">
         <v>7</v>
       </c>
-      <c r="B8" t="str">
+      <c r="C8" t="str">
         <v>QH Amateur Owner Performance Colt/Stallion</v>
       </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
       <c r="D8" t="str">
         <v/>
       </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="A9">
+      <c r="A9" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B9">
         <v>8</v>
       </c>
-      <c r="B9" t="str">
+      <c r="C9" t="str">
         <v>QH Champ &amp; Reserve Amateur Owner Colt/Stallion</v>
       </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
       <c r="D9" t="str">
         <v/>
       </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="A10">
+      <c r="A10" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B10">
         <v>9</v>
       </c>
-      <c r="B10" t="str">
+      <c r="C10" t="str">
         <v>QH Filly 1 year &amp; under</v>
       </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
       <c r="D10" t="str">
         <v/>
       </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
-      <c r="A11">
+      <c r="A11" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B11">
         <v>10</v>
       </c>
-      <c r="B11" t="str">
+      <c r="C11" t="str">
         <v>QH Filly 2 &amp; 3 years</v>
       </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
       <c r="D11" t="str">
         <v/>
       </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
-      <c r="A12">
+      <c r="A12" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B12">
         <v>11</v>
       </c>
-      <c r="B12" t="str">
+      <c r="C12" t="str">
         <v>QH Mare 4 yrs &amp; over</v>
       </c>
-      <c r="C12" t="str">
-        <v/>
-      </c>
       <c r="D12" t="str">
         <v/>
       </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13">
+      <c r="A13" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B13">
         <v>12</v>
       </c>
-      <c r="B13" t="str">
+      <c r="C13" t="str">
         <v>QH Champ &amp; Reserve Filly/Mare</v>
       </c>
-      <c r="C13" t="str">
-        <v/>
-      </c>
       <c r="D13" t="str">
         <v/>
       </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
-      <c r="A14">
+      <c r="A14" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B14">
         <v>13</v>
       </c>
-      <c r="B14" t="str">
+      <c r="C14" t="str">
         <v>QH Amateur Owner Filly 3 yrs &amp; under</v>
       </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
       <c r="D14" t="str">
         <v/>
       </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
-      <c r="A15">
+      <c r="A15" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B15">
         <v>14</v>
       </c>
-      <c r="B15" t="str">
+      <c r="C15" t="str">
         <v>QH Amateur Owner Mare 4 yrs &amp; over</v>
       </c>
-      <c r="C15" t="str">
-        <v/>
-      </c>
       <c r="D15" t="str">
         <v/>
       </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
-      <c r="A16">
+      <c r="A16" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B16">
         <v>15</v>
       </c>
-      <c r="B16" t="str">
+      <c r="C16" t="str">
         <v>QH Amateur Owner Performance Filly/Mare</v>
       </c>
-      <c r="C16" t="str">
-        <v/>
-      </c>
       <c r="D16" t="str">
         <v/>
       </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
-      <c r="A17">
+      <c r="A17" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B17">
         <v>16</v>
       </c>
-      <c r="B17" t="str">
+      <c r="C17" t="str">
         <v>QH Champ &amp; Reserve Amateur Owner Filly/Mare</v>
       </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
       <c r="D17" t="str">
         <v/>
       </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
-      <c r="A18">
+      <c r="A18" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B18">
         <v>17</v>
       </c>
-      <c r="B18" t="str">
+      <c r="C18" t="str">
         <v>QH Filly 2 yrs &amp; under YOUTH</v>
       </c>
-      <c r="C18" t="str">
-        <v/>
-      </c>
       <c r="D18" t="str">
         <v/>
       </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
-      <c r="A19">
+      <c r="A19" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B19">
         <v>18</v>
       </c>
-      <c r="B19" t="str">
+      <c r="C19" t="str">
         <v>QH Mare 3 yrs &amp; over YOUTH</v>
       </c>
-      <c r="C19" t="str">
-        <v/>
-      </c>
       <c r="D19" t="str">
         <v/>
       </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
-      <c r="A20">
+      <c r="A20" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B20">
         <v>19</v>
       </c>
-      <c r="B20" t="str">
+      <c r="C20" t="str">
         <v>QH Champ &amp; Reserve Filly/Mare YOUTH</v>
       </c>
-      <c r="C20" t="str">
-        <v/>
-      </c>
       <c r="D20" t="str">
         <v/>
       </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
-      <c r="A21">
+      <c r="A21" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B21">
         <v>20</v>
       </c>
-      <c r="B21" t="str">
+      <c r="C21" t="str">
         <v>QH Gelding 1 year &amp; under</v>
       </c>
-      <c r="C21" t="str">
-        <v/>
-      </c>
       <c r="D21" t="str">
         <v/>
       </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
-      <c r="A22">
+      <c r="A22" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B22">
         <v>21</v>
       </c>
-      <c r="B22" t="str">
+      <c r="C22" t="str">
         <v>QH Gelding 2 &amp; 3 years</v>
       </c>
-      <c r="C22" t="str">
-        <v/>
-      </c>
       <c r="D22" t="str">
         <v/>
       </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
-      <c r="A23">
+      <c r="A23" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B23">
         <v>22</v>
       </c>
-      <c r="B23" t="str">
+      <c r="C23" t="str">
         <v>QH Gelding 4 yrs &amp; over</v>
       </c>
-      <c r="C23" t="str">
-        <v/>
-      </c>
       <c r="D23" t="str">
         <v/>
       </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
-      <c r="A24">
+      <c r="A24" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B24">
         <v>23</v>
       </c>
-      <c r="B24" t="str">
+      <c r="C24" t="str">
         <v>QH Champ &amp; Reserve Gelding</v>
       </c>
-      <c r="C24" t="str">
-        <v/>
-      </c>
       <c r="D24" t="str">
         <v/>
       </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
-      <c r="A25">
+      <c r="A25" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B25">
         <v>24</v>
       </c>
-      <c r="B25" t="str">
+      <c r="C25" t="str">
         <v>QH Amateur Owner Gelding 3 yrs &amp; under</v>
       </c>
-      <c r="C25" t="str">
-        <v/>
-      </c>
       <c r="D25" t="str">
         <v/>
       </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
-      <c r="A26">
+      <c r="A26" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B26">
         <v>25</v>
       </c>
-      <c r="B26" t="str">
+      <c r="C26" t="str">
         <v>QH Amateur Owner Gelding 4 yrs &amp; over</v>
       </c>
-      <c r="C26" t="str">
-        <v/>
-      </c>
       <c r="D26" t="str">
         <v/>
       </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
-      <c r="A27">
+      <c r="A27" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B27">
         <v>26</v>
       </c>
-      <c r="B27" t="str">
+      <c r="C27" t="str">
         <v>QH Amateur Owner Performance Gelding</v>
       </c>
-      <c r="C27" t="str">
-        <v/>
-      </c>
       <c r="D27" t="str">
         <v/>
       </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
-      <c r="A28">
+      <c r="A28" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B28">
         <v>27</v>
       </c>
-      <c r="B28" t="str">
+      <c r="C28" t="str">
         <v>QH Champ &amp; Reserve Amateur Owner Gelding</v>
       </c>
-      <c r="C28" t="str">
-        <v/>
-      </c>
       <c r="D28" t="str">
         <v/>
       </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
-      <c r="A29">
+      <c r="A29" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B29">
         <v>28</v>
       </c>
-      <c r="B29" t="str">
+      <c r="C29" t="str">
         <v>QH Gelding 2 &amp; under YOUTH</v>
       </c>
-      <c r="C29" t="str">
-        <v/>
-      </c>
       <c r="D29" t="str">
         <v/>
       </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
-      <c r="A30">
+      <c r="A30" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B30">
         <v>29</v>
       </c>
-      <c r="B30" t="str">
+      <c r="C30" t="str">
         <v>QH Gelding 3 yrs &amp; over YOUTH</v>
       </c>
-      <c r="C30" t="str">
-        <v/>
-      </c>
       <c r="D30" t="str">
         <v/>
       </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
-      <c r="A31">
+      <c r="A31" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B31">
         <v>30</v>
       </c>
-      <c r="B31" t="str">
+      <c r="C31" t="str">
         <v>QH Champ &amp; Reserve Gelding YOUTH</v>
       </c>
-      <c r="C31" t="str">
-        <v/>
-      </c>
       <c r="D31" t="str">
         <v/>
       </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
-      <c r="A32">
+      <c r="A32" t="str">
+        <v>Quarter Horse Halter</v>
+      </c>
+      <c r="B32">
         <v>31</v>
       </c>
-      <c r="B32" t="str">
+      <c r="C32" t="str">
         <v>QH Grand Champion</v>
       </c>
-      <c r="C32" t="str">
-        <v/>
-      </c>
       <c r="D32" t="str">
         <v/>
       </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
-      <c r="A33">
+      <c r="A33" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B33">
         <v>32</v>
       </c>
-      <c r="B33" t="str">
+      <c r="C33" t="str">
         <v>Paint Colt 1 year &amp; under</v>
       </c>
-      <c r="C33" t="str">
-        <v/>
-      </c>
       <c r="D33" t="str">
         <v/>
       </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
-      <c r="A34">
+      <c r="A34" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B34">
         <v>33</v>
       </c>
-      <c r="B34" t="str">
+      <c r="C34" t="str">
         <v>Paint Colt 2 &amp; 3 years</v>
       </c>
-      <c r="C34" t="str">
-        <v/>
-      </c>
       <c r="D34" t="str">
         <v/>
       </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
-      <c r="A35">
+      <c r="A35" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B35">
         <v>34</v>
       </c>
-      <c r="B35" t="str">
+      <c r="C35" t="str">
         <v>Paint Stallion 4 yrs &amp; over</v>
       </c>
-      <c r="C35" t="str">
-        <v/>
-      </c>
       <c r="D35" t="str">
         <v/>
       </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
-      <c r="A36">
+      <c r="A36" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B36">
         <v>35</v>
       </c>
-      <c r="B36" t="str">
+      <c r="C36" t="str">
         <v>Paint Champ &amp; Reserve Colt/Stallion</v>
       </c>
-      <c r="C36" t="str">
-        <v/>
-      </c>
       <c r="D36" t="str">
         <v/>
       </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
-      <c r="A37">
+      <c r="A37" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B37">
         <v>36</v>
       </c>
-      <c r="B37" t="str">
+      <c r="C37" t="str">
         <v>Paint Amateur Owner Colt 3 yrs &amp; under</v>
       </c>
-      <c r="C37" t="str">
-        <v/>
-      </c>
       <c r="D37" t="str">
         <v/>
       </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
-      <c r="A38">
+      <c r="A38" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B38">
         <v>37</v>
       </c>
-      <c r="B38" t="str">
+      <c r="C38" t="str">
         <v>Paint Amateur Owner Stallion 4 yrs &amp; over</v>
       </c>
-      <c r="C38" t="str">
-        <v/>
-      </c>
       <c r="D38" t="str">
         <v/>
       </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
-      <c r="A39">
+      <c r="A39" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B39">
         <v>38</v>
       </c>
-      <c r="B39" t="str">
+      <c r="C39" t="str">
         <v>Paint Champ &amp; Reserve A/O Colt/Stallion</v>
       </c>
-      <c r="C39" t="str">
-        <v/>
-      </c>
       <c r="D39" t="str">
         <v/>
       </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
-      <c r="A40">
+      <c r="A40" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B40">
         <v>39</v>
       </c>
-      <c r="B40" t="str">
+      <c r="C40" t="str">
         <v>Paint Filly 1 year &amp; under</v>
       </c>
-      <c r="C40" t="str">
-        <v/>
-      </c>
       <c r="D40" t="str">
         <v/>
       </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
-      <c r="A41">
+      <c r="A41" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B41">
         <v>40</v>
       </c>
-      <c r="B41" t="str">
+      <c r="C41" t="str">
         <v>Paint Filly 2 &amp; 3 years</v>
       </c>
-      <c r="C41" t="str">
-        <v/>
-      </c>
       <c r="D41" t="str">
         <v/>
       </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
-      <c r="A42">
+      <c r="A42" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B42">
         <v>41</v>
       </c>
-      <c r="B42" t="str">
+      <c r="C42" t="str">
         <v>Paint Mare 4 yrs &amp; over</v>
       </c>
-      <c r="C42" t="str">
-        <v/>
-      </c>
       <c r="D42" t="str">
         <v/>
       </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
-      <c r="A43">
+      <c r="A43" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B43">
         <v>42</v>
       </c>
-      <c r="B43" t="str">
+      <c r="C43" t="str">
         <v>Paint Champ &amp; Reserve Filly/Mare</v>
       </c>
-      <c r="C43" t="str">
-        <v/>
-      </c>
       <c r="D43" t="str">
         <v/>
       </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
-      <c r="A44">
+      <c r="A44" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B44">
         <v>43</v>
       </c>
-      <c r="B44" t="str">
+      <c r="C44" t="str">
         <v>Paint Amateur Owner Filly 3 yrs &amp; under</v>
       </c>
-      <c r="C44" t="str">
-        <v/>
-      </c>
       <c r="D44" t="str">
         <v/>
       </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
-      <c r="A45">
+      <c r="A45" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B45">
         <v>44</v>
       </c>
-      <c r="B45" t="str">
+      <c r="C45" t="str">
         <v>Paint Amateur Owner Mare 4 yrs &amp; over</v>
       </c>
-      <c r="C45" t="str">
-        <v/>
-      </c>
       <c r="D45" t="str">
         <v/>
       </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
-      <c r="A46">
+      <c r="A46" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B46">
         <v>45</v>
       </c>
-      <c r="B46" t="str">
+      <c r="C46" t="str">
         <v>Paint Champ &amp; Reserve A/O Filly/Mare</v>
       </c>
-      <c r="C46" t="str">
-        <v/>
-      </c>
       <c r="D46" t="str">
         <v/>
       </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
-      <c r="A47">
+      <c r="A47" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B47">
         <v>46</v>
       </c>
-      <c r="B47" t="str">
+      <c r="C47" t="str">
         <v>Paint Filly 2 yrs &amp; under YOUTH</v>
       </c>
-      <c r="C47" t="str">
-        <v/>
-      </c>
       <c r="D47" t="str">
         <v/>
       </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
-      <c r="A48">
+      <c r="A48" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B48">
         <v>47</v>
       </c>
-      <c r="B48" t="str">
+      <c r="C48" t="str">
         <v>Paint Mare 3 yrs &amp; over YOUTH</v>
       </c>
-      <c r="C48" t="str">
-        <v/>
-      </c>
       <c r="D48" t="str">
         <v/>
       </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
-      <c r="A49">
+      <c r="A49" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B49">
         <v>48</v>
       </c>
-      <c r="B49" t="str">
+      <c r="C49" t="str">
         <v>Paint Champ &amp; Reserve Filly/Mare YOUTH</v>
       </c>
-      <c r="C49" t="str">
-        <v/>
-      </c>
       <c r="D49" t="str">
         <v/>
       </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
-      <c r="A50">
+      <c r="A50" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B50">
         <v>49</v>
       </c>
-      <c r="B50" t="str">
+      <c r="C50" t="str">
         <v>Paint Gelding 1 year &amp; under</v>
       </c>
-      <c r="C50" t="str">
-        <v/>
-      </c>
       <c r="D50" t="str">
         <v/>
       </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
-      <c r="A51">
+      <c r="A51" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B51">
         <v>50</v>
       </c>
-      <c r="B51" t="str">
+      <c r="C51" t="str">
         <v>Paint Gelding 2 &amp; 3 years</v>
       </c>
-      <c r="C51" t="str">
-        <v/>
-      </c>
       <c r="D51" t="str">
         <v/>
       </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
-      <c r="A52">
+      <c r="A52" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B52">
         <v>51</v>
       </c>
-      <c r="B52" t="str">
+      <c r="C52" t="str">
         <v>Paint Gelding 4 yrs &amp; over</v>
       </c>
-      <c r="C52" t="str">
-        <v/>
-      </c>
       <c r="D52" t="str">
         <v/>
       </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
-      <c r="A53">
+      <c r="A53" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B53">
         <v>52</v>
       </c>
-      <c r="B53" t="str">
+      <c r="C53" t="str">
         <v>Paint Champ &amp; Reserve Gelding</v>
       </c>
-      <c r="C53" t="str">
-        <v/>
-      </c>
       <c r="D53" t="str">
         <v/>
       </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
-      <c r="A54">
+      <c r="A54" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B54">
         <v>53</v>
       </c>
-      <c r="B54" t="str">
+      <c r="C54" t="str">
         <v>Paint Amateur Owner Gelding 3 yrs &amp; under</v>
       </c>
-      <c r="C54" t="str">
-        <v/>
-      </c>
       <c r="D54" t="str">
         <v/>
       </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
-      <c r="A55">
+      <c r="A55" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B55">
         <v>54</v>
       </c>
-      <c r="B55" t="str">
+      <c r="C55" t="str">
         <v>Paint Amateur Owner Gelding 4 yrs &amp; over</v>
       </c>
-      <c r="C55" t="str">
-        <v/>
-      </c>
       <c r="D55" t="str">
         <v/>
       </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
-      <c r="A56">
+      <c r="A56" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B56">
         <v>55</v>
       </c>
-      <c r="B56" t="str">
+      <c r="C56" t="str">
         <v>Paint Champ &amp; Reserve A/O Gelding</v>
       </c>
-      <c r="C56" t="str">
-        <v/>
-      </c>
       <c r="D56" t="str">
         <v/>
       </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
-      <c r="A57">
+      <c r="A57" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B57">
         <v>56</v>
       </c>
-      <c r="B57" t="str">
+      <c r="C57" t="str">
         <v>Paint Gelding 2 &amp; under YOUTH</v>
       </c>
-      <c r="C57" t="str">
-        <v/>
-      </c>
       <c r="D57" t="str">
         <v/>
       </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
-      <c r="A58">
+      <c r="A58" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B58">
         <v>57</v>
       </c>
-      <c r="B58" t="str">
+      <c r="C58" t="str">
         <v>Paint Gelding 3 yrs &amp; over YOUTH</v>
       </c>
-      <c r="C58" t="str">
-        <v/>
-      </c>
       <c r="D58" t="str">
         <v/>
       </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
-      <c r="A59">
+      <c r="A59" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B59">
         <v>58</v>
       </c>
-      <c r="B59" t="str">
+      <c r="C59" t="str">
         <v>Paint Champ &amp; Reserve Gelding YOUTH</v>
       </c>
-      <c r="C59" t="str">
-        <v/>
-      </c>
       <c r="D59" t="str">
         <v/>
       </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
-      <c r="A60">
+      <c r="A60" t="str">
+        <v>Paint Halter</v>
+      </c>
+      <c r="B60">
         <v>59</v>
       </c>
-      <c r="B60" t="str">
+      <c r="C60" t="str">
         <v>Paint Grand Champion</v>
       </c>
-      <c r="C60" t="str">
-        <v/>
-      </c>
       <c r="D60" t="str">
         <v/>
       </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
-      <c r="A61">
+      <c r="A61" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B61">
         <v>60</v>
       </c>
-      <c r="B61" t="str">
+      <c r="C61" t="str">
         <v>Paint Bred Colt 1 year &amp; under</v>
       </c>
-      <c r="C61" t="str">
-        <v/>
-      </c>
       <c r="D61" t="str">
         <v/>
       </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
-      <c r="A62">
+      <c r="A62" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B62">
         <v>61</v>
       </c>
-      <c r="B62" t="str">
+      <c r="C62" t="str">
         <v>Paint Bred Colt 2 &amp; 3 years</v>
       </c>
-      <c r="C62" t="str">
-        <v/>
-      </c>
       <c r="D62" t="str">
         <v/>
       </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
-      <c r="A63">
+      <c r="A63" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B63">
         <v>62</v>
       </c>
-      <c r="B63" t="str">
+      <c r="C63" t="str">
         <v>Paint Bred Stallion 4 yrs &amp; over</v>
       </c>
-      <c r="C63" t="str">
-        <v/>
-      </c>
       <c r="D63" t="str">
         <v/>
       </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
-      <c r="A64">
+      <c r="A64" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B64">
         <v>63</v>
       </c>
-      <c r="B64" t="str">
+      <c r="C64" t="str">
         <v>Paint Bred Champ &amp; Reserve Colt/Stallion</v>
       </c>
-      <c r="C64" t="str">
-        <v/>
-      </c>
       <c r="D64" t="str">
         <v/>
       </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
-      <c r="A65">
+      <c r="A65" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B65">
         <v>64</v>
       </c>
-      <c r="B65" t="str">
+      <c r="C65" t="str">
         <v>Paint Bred Amateur Owner Colt 3 yrs &amp; under</v>
       </c>
-      <c r="C65" t="str">
-        <v/>
-      </c>
       <c r="D65" t="str">
         <v/>
       </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
-      <c r="A66">
+      <c r="A66" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B66">
         <v>65</v>
       </c>
-      <c r="B66" t="str">
+      <c r="C66" t="str">
         <v>Paint Bred Amateur Owner Stallion 4 yrs &amp; over</v>
       </c>
-      <c r="C66" t="str">
-        <v/>
-      </c>
       <c r="D66" t="str">
         <v/>
       </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
-      <c r="A67">
+      <c r="A67" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B67">
         <v>66</v>
       </c>
-      <c r="B67" t="str">
+      <c r="C67" t="str">
         <v>Paint Bred Champ &amp; Reserve A/O Colt/Stallion</v>
       </c>
-      <c r="C67" t="str">
-        <v/>
-      </c>
       <c r="D67" t="str">
         <v/>
       </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
-      <c r="A68">
+      <c r="A68" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B68">
         <v>67</v>
       </c>
-      <c r="B68" t="str">
+      <c r="C68" t="str">
         <v>Paint Bred Filly 1 year &amp; under</v>
       </c>
-      <c r="C68" t="str">
-        <v/>
-      </c>
       <c r="D68" t="str">
         <v/>
       </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
-      <c r="A69">
+      <c r="A69" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B69">
         <v>68</v>
       </c>
-      <c r="B69" t="str">
+      <c r="C69" t="str">
         <v>Paint Bred Filly 2 &amp; 3 years</v>
       </c>
-      <c r="C69" t="str">
-        <v/>
-      </c>
       <c r="D69" t="str">
         <v/>
       </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
-      <c r="A70">
+      <c r="A70" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B70">
         <v>69</v>
       </c>
-      <c r="B70" t="str">
+      <c r="C70" t="str">
         <v>Paint Bred Mare 4 yrs &amp; over</v>
       </c>
-      <c r="C70" t="str">
-        <v/>
-      </c>
       <c r="D70" t="str">
         <v/>
       </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
-      <c r="A71">
+      <c r="A71" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B71">
         <v>70</v>
       </c>
-      <c r="B71" t="str">
+      <c r="C71" t="str">
         <v>Paint Bred Champ &amp; Reserve Filly/Mare</v>
       </c>
-      <c r="C71" t="str">
-        <v/>
-      </c>
       <c r="D71" t="str">
         <v/>
       </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
-      <c r="A72">
+      <c r="A72" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B72">
         <v>71</v>
       </c>
-      <c r="B72" t="str">
+      <c r="C72" t="str">
         <v>Paint Bred Amateur Owner Filly 3 yrs &amp; under</v>
       </c>
-      <c r="C72" t="str">
-        <v/>
-      </c>
       <c r="D72" t="str">
         <v/>
       </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
-      <c r="A73">
+      <c r="A73" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B73">
         <v>72</v>
       </c>
-      <c r="B73" t="str">
+      <c r="C73" t="str">
         <v>Paint Bred Amateur Owner Mare 4 yrs &amp; over</v>
       </c>
-      <c r="C73" t="str">
-        <v/>
-      </c>
       <c r="D73" t="str">
         <v/>
       </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
-      <c r="A74">
+      <c r="A74" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B74">
         <v>73</v>
       </c>
-      <c r="B74" t="str">
+      <c r="C74" t="str">
         <v>Paint Bred Champ &amp; Reserve A/O Filly/Mare</v>
       </c>
-      <c r="C74" t="str">
-        <v/>
-      </c>
       <c r="D74" t="str">
         <v/>
       </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
-      <c r="A75">
+      <c r="A75" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B75">
         <v>74</v>
       </c>
-      <c r="B75" t="str">
+      <c r="C75" t="str">
         <v>Paint Bred Filly 2 yrs &amp; under YOUTH</v>
       </c>
-      <c r="C75" t="str">
-        <v/>
-      </c>
       <c r="D75" t="str">
         <v/>
       </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
-      <c r="A76">
+      <c r="A76" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B76">
         <v>75</v>
       </c>
-      <c r="B76" t="str">
+      <c r="C76" t="str">
         <v>Paint Bred Mare 3 yrs &amp; over YOUTH</v>
       </c>
-      <c r="C76" t="str">
-        <v/>
-      </c>
       <c r="D76" t="str">
         <v/>
       </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
-      <c r="A77">
+      <c r="A77" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B77">
         <v>76</v>
       </c>
-      <c r="B77" t="str">
+      <c r="C77" t="str">
         <v>Paint Bred Champ &amp; Reserve Filly/Mare YOUTH</v>
       </c>
-      <c r="C77" t="str">
-        <v/>
-      </c>
       <c r="D77" t="str">
         <v/>
       </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
-      <c r="A78">
+      <c r="A78" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B78">
         <v>77</v>
       </c>
-      <c r="B78" t="str">
+      <c r="C78" t="str">
         <v>Paint Bred Gelding 1 year &amp; under</v>
       </c>
-      <c r="C78" t="str">
-        <v/>
-      </c>
       <c r="D78" t="str">
         <v/>
       </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
-      <c r="A79">
+      <c r="A79" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B79">
         <v>78</v>
       </c>
-      <c r="B79" t="str">
+      <c r="C79" t="str">
         <v>Paint Bred Gelding 2 &amp; 3 years</v>
       </c>
-      <c r="C79" t="str">
-        <v/>
-      </c>
       <c r="D79" t="str">
         <v/>
       </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
-      <c r="A80">
+      <c r="A80" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B80">
         <v>79</v>
       </c>
-      <c r="B80" t="str">
+      <c r="C80" t="str">
         <v>Paint Bred Gelding 4 yrs &amp; over</v>
       </c>
-      <c r="C80" t="str">
-        <v/>
-      </c>
       <c r="D80" t="str">
         <v/>
       </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
-      <c r="A81">
+      <c r="A81" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B81">
         <v>80</v>
       </c>
-      <c r="B81" t="str">
+      <c r="C81" t="str">
         <v>Paint Bred Champ &amp; Reserve Gelding</v>
       </c>
-      <c r="C81" t="str">
-        <v/>
-      </c>
       <c r="D81" t="str">
         <v/>
       </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
-      <c r="A82">
+      <c r="A82" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B82">
         <v>81</v>
       </c>
-      <c r="B82" t="str">
+      <c r="C82" t="str">
         <v>Paint Bred Amateur Owner Gelding 3 yrs &amp; under</v>
       </c>
-      <c r="C82" t="str">
-        <v/>
-      </c>
       <c r="D82" t="str">
         <v/>
       </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
-      <c r="A83">
+      <c r="A83" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B83">
         <v>82</v>
       </c>
-      <c r="B83" t="str">
+      <c r="C83" t="str">
         <v>Paint Bred Amateur Owner Gelding 4 yrs &amp; over</v>
       </c>
-      <c r="C83" t="str">
-        <v/>
-      </c>
       <c r="D83" t="str">
         <v/>
       </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
-      <c r="A84">
+      <c r="A84" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B84">
         <v>83</v>
       </c>
-      <c r="B84" t="str">
+      <c r="C84" t="str">
         <v>Paint Bred Champ &amp; Reserve A/O Gelding</v>
       </c>
-      <c r="C84" t="str">
-        <v/>
-      </c>
       <c r="D84" t="str">
         <v/>
       </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
-      <c r="A85">
+      <c r="A85" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B85">
         <v>84</v>
       </c>
-      <c r="B85" t="str">
+      <c r="C85" t="str">
         <v>Paint Bred Gelding 2 &amp; under YOUTH</v>
       </c>
-      <c r="C85" t="str">
-        <v/>
-      </c>
       <c r="D85" t="str">
         <v/>
       </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
-      <c r="A86">
+      <c r="A86" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B86">
         <v>85</v>
       </c>
-      <c r="B86" t="str">
+      <c r="C86" t="str">
         <v>Paint Bred Gelding 3 yrs &amp; over YOUTH</v>
       </c>
-      <c r="C86" t="str">
-        <v/>
-      </c>
       <c r="D86" t="str">
         <v/>
       </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
-      <c r="A87">
+      <c r="A87" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B87">
         <v>86</v>
       </c>
-      <c r="B87" t="str">
+      <c r="C87" t="str">
         <v>Paint Bred Champ &amp; Reserve Gelding YOUTH</v>
       </c>
-      <c r="C87" t="str">
-        <v/>
-      </c>
       <c r="D87" t="str">
         <v/>
       </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
-      <c r="A88">
+      <c r="A88" t="str">
+        <v>Paint Bred Halter</v>
+      </c>
+      <c r="B88">
         <v>87</v>
       </c>
-      <c r="B88" t="str">
+      <c r="C88" t="str">
         <v>Paint Bred Grand Champion</v>
       </c>
-      <c r="C88" t="str">
-        <v/>
-      </c>
       <c r="D88" t="str">
         <v/>
       </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
-      <c r="A89">
+      <c r="A89" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B89">
         <v>88</v>
       </c>
-      <c r="B89" t="str">
+      <c r="C89" t="str">
         <v>Appaloosa Colt 1 year &amp; under</v>
       </c>
-      <c r="C89" t="str">
-        <v/>
-      </c>
       <c r="D89" t="str">
         <v/>
       </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
-      <c r="A90">
+      <c r="A90" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B90">
         <v>89</v>
       </c>
-      <c r="B90" t="str">
+      <c r="C90" t="str">
         <v>Appaloosa Colt 2 &amp; 3 years</v>
       </c>
-      <c r="C90" t="str">
-        <v/>
-      </c>
       <c r="D90" t="str">
         <v/>
       </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
-      <c r="A91">
+      <c r="A91" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B91">
         <v>90</v>
       </c>
-      <c r="B91" t="str">
+      <c r="C91" t="str">
         <v>Appaloosa Stallion 4 yrs &amp; over</v>
       </c>
-      <c r="C91" t="str">
-        <v/>
-      </c>
       <c r="D91" t="str">
         <v/>
       </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
-      <c r="A92">
+      <c r="A92" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B92">
         <v>91</v>
       </c>
-      <c r="B92" t="str">
+      <c r="C92" t="str">
         <v>Appaloosa Champ &amp; Reserve Colt/Stallion</v>
       </c>
-      <c r="C92" t="str">
-        <v/>
-      </c>
       <c r="D92" t="str">
         <v/>
       </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
-      <c r="A93">
+      <c r="A93" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B93">
         <v>92</v>
       </c>
-      <c r="B93" t="str">
+      <c r="C93" t="str">
         <v>Appaloosa Amateur Owner Colt 3 yrs &amp; under</v>
       </c>
-      <c r="C93" t="str">
-        <v/>
-      </c>
       <c r="D93" t="str">
         <v/>
       </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
-      <c r="A94">
+      <c r="A94" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B94">
         <v>93</v>
       </c>
-      <c r="B94" t="str">
+      <c r="C94" t="str">
         <v>Appaloosa Amateur Owner Stallion 4 yrs &amp; over</v>
       </c>
-      <c r="C94" t="str">
-        <v/>
-      </c>
       <c r="D94" t="str">
         <v/>
       </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
-      <c r="A95">
+      <c r="A95" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B95">
         <v>94</v>
       </c>
-      <c r="B95" t="str">
+      <c r="C95" t="str">
         <v>Appaloosa Champ &amp; Reserve A/O Colt/Stallion</v>
       </c>
-      <c r="C95" t="str">
-        <v/>
-      </c>
       <c r="D95" t="str">
         <v/>
       </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
-      <c r="A96">
+      <c r="A96" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B96">
         <v>95</v>
       </c>
-      <c r="B96" t="str">
+      <c r="C96" t="str">
         <v>Appaloosa Filly 1 year &amp; under</v>
       </c>
-      <c r="C96" t="str">
-        <v/>
-      </c>
       <c r="D96" t="str">
         <v/>
       </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
     </row>
     <row r="97">
-      <c r="A97">
+      <c r="A97" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B97">
         <v>96</v>
       </c>
-      <c r="B97" t="str">
+      <c r="C97" t="str">
         <v>Appaloosa Filly 2 &amp; 3 years</v>
       </c>
-      <c r="C97" t="str">
-        <v/>
-      </c>
       <c r="D97" t="str">
         <v/>
       </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
-      <c r="A98">
+      <c r="A98" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B98">
         <v>97</v>
       </c>
-      <c r="B98" t="str">
+      <c r="C98" t="str">
         <v>Appaloosa Mare 4 yrs &amp; over</v>
       </c>
-      <c r="C98" t="str">
-        <v/>
-      </c>
       <c r="D98" t="str">
         <v/>
       </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
-      <c r="A99">
+      <c r="A99" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B99">
         <v>98</v>
       </c>
-      <c r="B99" t="str">
+      <c r="C99" t="str">
         <v>Appaloosa Champ &amp; Reserve Filly/Mare</v>
       </c>
-      <c r="C99" t="str">
-        <v/>
-      </c>
       <c r="D99" t="str">
         <v/>
       </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
     </row>
     <row r="100">
-      <c r="A100">
+      <c r="A100" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B100">
         <v>99</v>
       </c>
-      <c r="B100" t="str">
+      <c r="C100" t="str">
         <v>Appaloosa Amateur Owner Filly 3 yrs &amp; under</v>
       </c>
-      <c r="C100" t="str">
-        <v/>
-      </c>
       <c r="D100" t="str">
         <v/>
       </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
-      <c r="A101">
+      <c r="A101" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B101">
         <v>100</v>
       </c>
-      <c r="B101" t="str">
+      <c r="C101" t="str">
         <v>Appaloosa Amateur Owner Mare 4 yrs &amp; over</v>
       </c>
-      <c r="C101" t="str">
-        <v/>
-      </c>
       <c r="D101" t="str">
         <v/>
       </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
     </row>
     <row r="102">
-      <c r="A102">
+      <c r="A102" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B102">
         <v>101</v>
       </c>
-      <c r="B102" t="str">
+      <c r="C102" t="str">
         <v>Appaloosa Champ &amp; Reserve A/O Filly/Mare</v>
       </c>
-      <c r="C102" t="str">
-        <v/>
-      </c>
       <c r="D102" t="str">
         <v/>
       </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
     </row>
     <row r="103">
-      <c r="A103">
+      <c r="A103" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B103">
         <v>102</v>
       </c>
-      <c r="B103" t="str">
+      <c r="C103" t="str">
         <v>Appaloosa Gelding 1 year &amp; under</v>
       </c>
-      <c r="C103" t="str">
-        <v/>
-      </c>
       <c r="D103" t="str">
         <v/>
       </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
     </row>
     <row r="104">
-      <c r="A104">
+      <c r="A104" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B104">
         <v>103</v>
       </c>
-      <c r="B104" t="str">
+      <c r="C104" t="str">
         <v>Appaloosa Gelding 2 &amp; 3 years</v>
       </c>
-      <c r="C104" t="str">
-        <v/>
-      </c>
       <c r="D104" t="str">
         <v/>
       </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
     </row>
     <row r="105">
-      <c r="A105">
+      <c r="A105" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B105">
         <v>104</v>
       </c>
-      <c r="B105" t="str">
+      <c r="C105" t="str">
         <v>Appaloosa Gelding 4 yrs &amp; over</v>
       </c>
-      <c r="C105" t="str">
-        <v/>
-      </c>
       <c r="D105" t="str">
         <v/>
       </c>
+      <c r="E105" t="str">
+        <v/>
+      </c>
     </row>
     <row r="106">
-      <c r="A106">
+      <c r="A106" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B106">
         <v>105</v>
       </c>
-      <c r="B106" t="str">
+      <c r="C106" t="str">
         <v>Appaloosa Champ &amp; Reserve Gelding</v>
       </c>
-      <c r="C106" t="str">
-        <v/>
-      </c>
       <c r="D106" t="str">
         <v/>
       </c>
+      <c r="E106" t="str">
+        <v/>
+      </c>
     </row>
     <row r="107">
-      <c r="A107">
+      <c r="A107" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B107">
         <v>106</v>
       </c>
-      <c r="B107" t="str">
+      <c r="C107" t="str">
         <v>Appaloosa Amateur Owner Gelding 3 yrs &amp; under</v>
       </c>
-      <c r="C107" t="str">
-        <v/>
-      </c>
       <c r="D107" t="str">
         <v/>
       </c>
+      <c r="E107" t="str">
+        <v/>
+      </c>
     </row>
     <row r="108">
-      <c r="A108">
+      <c r="A108" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B108">
         <v>107</v>
       </c>
-      <c r="B108" t="str">
+      <c r="C108" t="str">
         <v>Appaloosa Amateur Owner Gelding 4 yrs &amp; over</v>
       </c>
-      <c r="C108" t="str">
-        <v/>
-      </c>
       <c r="D108" t="str">
         <v/>
       </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
     </row>
     <row r="109">
-      <c r="A109">
+      <c r="A109" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B109">
         <v>108</v>
       </c>
-      <c r="B109" t="str">
+      <c r="C109" t="str">
         <v>Appaloosa Champ &amp; Reserve A/O Gelding</v>
       </c>
-      <c r="C109" t="str">
-        <v/>
-      </c>
       <c r="D109" t="str">
         <v/>
       </c>
+      <c r="E109" t="str">
+        <v/>
+      </c>
     </row>
     <row r="110">
-      <c r="A110">
+      <c r="A110" t="str">
+        <v>Appaloosa Halter</v>
+      </c>
+      <c r="B110">
         <v>109</v>
       </c>
-      <c r="B110" t="str">
+      <c r="C110" t="str">
         <v>Appaloosa Grand Champion</v>
       </c>
-      <c r="C110" t="str">
-        <v/>
-      </c>
       <c r="D110" t="str">
         <v/>
       </c>
+      <c r="E110" t="str">
+        <v/>
+      </c>
     </row>
     <row r="111">
-      <c r="A111">
+      <c r="A111" t="str">
+        <v>Other Breeds Halter</v>
+      </c>
+      <c r="B111">
         <v>110</v>
       </c>
-      <c r="B111" t="str">
+      <c r="C111" t="str">
         <v>Other Breeds Halter</v>
       </c>
-      <c r="C111" t="str">
-        <v/>
-      </c>
       <c r="D111" t="str">
         <v/>
       </c>
+      <c r="E111" t="str">
+        <v/>
+      </c>
     </row>
     <row r="112">
-      <c r="A112">
+      <c r="A112" t="str">
+        <v>Other Breeds Halter</v>
+      </c>
+      <c r="B112">
         <v>111</v>
       </c>
-      <c r="B112" t="str">
+      <c r="C112" t="str">
         <v>Other Breeds Filly/Mare</v>
       </c>
-      <c r="C112" t="str">
-        <v/>
-      </c>
       <c r="D112" t="str">
         <v/>
       </c>
+      <c r="E112" t="str">
+        <v/>
+      </c>
     </row>
     <row r="113">
-      <c r="A113">
+      <c r="A113" t="str">
+        <v>Other Breeds Halter</v>
+      </c>
+      <c r="B113">
         <v>112</v>
       </c>
-      <c r="B113" t="str">
+      <c r="C113" t="str">
         <v>Other Breeds Colt/Stallion</v>
       </c>
-      <c r="C113" t="str">
-        <v/>
-      </c>
       <c r="D113" t="str">
         <v/>
       </c>
+      <c r="E113" t="str">
+        <v/>
+      </c>
     </row>
     <row r="114">
-      <c r="A114">
+      <c r="A114" t="str">
+        <v>Other Breeds Halter</v>
+      </c>
+      <c r="B114">
         <v>113</v>
       </c>
-      <c r="B114" t="str">
+      <c r="C114" t="str">
         <v>Other Breeds Gelding</v>
       </c>
-      <c r="C114" t="str">
-        <v/>
-      </c>
       <c r="D114" t="str">
         <v/>
       </c>
+      <c r="E114" t="str">
+        <v/>
+      </c>
     </row>
     <row r="115">
-      <c r="A115">
+      <c r="A115" t="str">
+        <v>Other Breeds Halter</v>
+      </c>
+      <c r="B115">
         <v>114</v>
       </c>
-      <c r="B115" t="str">
+      <c r="C115" t="str">
         <v>Other Breeds Grand Champion</v>
       </c>
-      <c r="C115" t="str">
-        <v/>
-      </c>
       <c r="D115" t="str">
         <v/>
       </c>
+      <c r="E115" t="str">
+        <v/>
+      </c>
     </row>
     <row r="116">
-      <c r="A116">
+      <c r="A116" t="str">
+        <v>Other Breeds Halter</v>
+      </c>
+      <c r="B116">
         <v>115</v>
       </c>
-      <c r="B116" t="str">
+      <c r="C116" t="str">
         <v>Supreme Halter Horse</v>
       </c>
-      <c r="C116" t="str">
-        <v/>
-      </c>
       <c r="D116" t="str">
         <v/>
       </c>
+      <c r="E116" t="str">
+        <v/>
+      </c>
     </row>
     <row r="117">
-      <c r="A117">
+      <c r="A117" t="str">
+        <v>Showmanship</v>
+      </c>
+      <c r="B117">
         <v>116</v>
       </c>
-      <c r="B117" t="str">
+      <c r="C117" t="str">
         <v>Amateur Showmanship</v>
       </c>
-      <c r="C117" t="str">
-        <v/>
-      </c>
       <c r="D117" t="str">
         <v/>
       </c>
+      <c r="E117" t="str">
+        <v/>
+      </c>
     </row>
     <row r="118">
-      <c r="A118">
+      <c r="A118" t="str">
+        <v>Showmanship</v>
+      </c>
+      <c r="B118">
         <v>117</v>
       </c>
-      <c r="B118" t="str">
+      <c r="C118" t="str">
         <v>Select Amateur Showmanship</v>
       </c>
-      <c r="C118" t="str">
-        <v/>
-      </c>
       <c r="D118" t="str">
         <v/>
       </c>
+      <c r="E118" t="str">
+        <v/>
+      </c>
     </row>
     <row r="119">
-      <c r="A119">
+      <c r="A119" t="str">
+        <v>Showmanship</v>
+      </c>
+      <c r="B119">
         <v>118</v>
       </c>
-      <c r="B119" t="str">
+      <c r="C119" t="str">
         <v>Novice Amateur Showmanship</v>
       </c>
-      <c r="C119" t="str">
-        <v/>
-      </c>
       <c r="D119" t="str">
         <v/>
       </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
     </row>
     <row r="120">
-      <c r="A120">
+      <c r="A120" t="str">
+        <v>Showmanship</v>
+      </c>
+      <c r="B120">
         <v>119</v>
       </c>
-      <c r="B120" t="str">
+      <c r="C120" t="str">
         <v>Beginner Showmanship</v>
       </c>
-      <c r="C120" t="str">
-        <v/>
-      </c>
       <c r="D120" t="str">
         <v/>
       </c>
+      <c r="E120" t="str">
+        <v/>
+      </c>
     </row>
     <row r="121">
-      <c r="A121">
+      <c r="A121" t="str">
+        <v>Showmanship</v>
+      </c>
+      <c r="B121">
         <v>120</v>
       </c>
-      <c r="B121" t="str">
+      <c r="C121" t="str">
         <v>Youth 5-11 yrs Showmanship</v>
       </c>
-      <c r="C121" t="str">
-        <v/>
-      </c>
       <c r="D121" t="str">
         <v/>
       </c>
+      <c r="E121" t="str">
+        <v/>
+      </c>
     </row>
     <row r="122">
-      <c r="A122">
+      <c r="A122" t="str">
+        <v>Showmanship</v>
+      </c>
+      <c r="B122">
         <v>121</v>
       </c>
-      <c r="B122" t="str">
+      <c r="C122" t="str">
         <v>Youth 12-14 yrs Showmanship</v>
       </c>
-      <c r="C122" t="str">
-        <v/>
-      </c>
       <c r="D122" t="str">
         <v/>
       </c>
+      <c r="E122" t="str">
+        <v/>
+      </c>
     </row>
     <row r="123">
-      <c r="A123">
+      <c r="A123" t="str">
+        <v>Showmanship</v>
+      </c>
+      <c r="B123">
         <v>122</v>
       </c>
-      <c r="B123" t="str">
+      <c r="C123" t="str">
         <v>Youth 15-18 yrs Showmanship</v>
       </c>
-      <c r="C123" t="str">
-        <v/>
-      </c>
       <c r="D123" t="str">
         <v/>
       </c>
+      <c r="E123" t="str">
+        <v/>
+      </c>
     </row>
     <row r="124">
-      <c r="A124">
+      <c r="A124" t="str">
+        <v>Showmanship</v>
+      </c>
+      <c r="B124">
         <v>123</v>
       </c>
-      <c r="B124" t="str">
+      <c r="C124" t="str">
         <v>EWD Showmanship</v>
       </c>
-      <c r="C124" t="str">
-        <v/>
-      </c>
       <c r="D124" t="str">
         <v/>
       </c>
+      <c r="E124" t="str">
+        <v/>
+      </c>
     </row>
     <row r="125">
-      <c r="A125">
+      <c r="A125" t="str">
+        <v>Lungeline</v>
+      </c>
+      <c r="B125">
         <v>124</v>
       </c>
-      <c r="B125" t="str">
+      <c r="C125" t="str">
         <v>Lungeline Yearling</v>
       </c>
-      <c r="C125" t="str">
-        <v/>
-      </c>
       <c r="D125" t="str">
         <v/>
       </c>
+      <c r="E125" t="str">
+        <v/>
+      </c>
     </row>
     <row r="126">
-      <c r="A126">
+      <c r="A126" t="str">
+        <v>Lungeline</v>
+      </c>
+      <c r="B126">
         <v>125</v>
       </c>
-      <c r="B126" t="str">
+      <c r="C126" t="str">
         <v>Lungeline 3 yrs &amp; over Versatility</v>
       </c>
-      <c r="C126" t="str">
-        <v/>
-      </c>
       <c r="D126" t="str">
         <v/>
       </c>
+      <c r="E126" t="str">
+        <v/>
+      </c>
     </row>
     <row r="127">
-      <c r="A127">
+      <c r="A127" t="str">
+        <v>Lungeline</v>
+      </c>
+      <c r="B127">
         <v>126</v>
       </c>
-      <c r="B127" t="str">
+      <c r="C127" t="str">
         <v>Lungeline 2 yr old</v>
       </c>
-      <c r="C127" t="str">
-        <v/>
-      </c>
       <c r="D127" t="str">
         <v/>
       </c>
+      <c r="E127" t="str">
+        <v/>
+      </c>
     </row>
     <row r="128">
-      <c r="A128">
+      <c r="A128" t="str">
+        <v>Hunter in Hand</v>
+      </c>
+      <c r="B128">
         <v>127</v>
       </c>
-      <c r="B128" t="str">
+      <c r="C128" t="str">
         <v>Hunter in Hand Yearling</v>
       </c>
-      <c r="C128" t="str">
-        <v/>
-      </c>
       <c r="D128" t="str">
         <v/>
       </c>
+      <c r="E128" t="str">
+        <v/>
+      </c>
     </row>
     <row r="129">
-      <c r="A129">
+      <c r="A129" t="str">
+        <v>Hunter in Hand</v>
+      </c>
+      <c r="B129">
         <v>128</v>
       </c>
-      <c r="B129" t="str">
+      <c r="C129" t="str">
         <v>Hunter in Hand 3 yrs &amp; over Versatility</v>
       </c>
-      <c r="C129" t="str">
-        <v/>
-      </c>
       <c r="D129" t="str">
         <v/>
       </c>
+      <c r="E129" t="str">
+        <v/>
+      </c>
     </row>
     <row r="130">
-      <c r="A130">
+      <c r="A130" t="str">
+        <v>Hunter in Hand</v>
+      </c>
+      <c r="B130">
         <v>129</v>
       </c>
-      <c r="B130" t="str">
+      <c r="C130" t="str">
         <v>Hunter in Hand 2 yr old &amp; over</v>
       </c>
-      <c r="C130" t="str">
-        <v/>
-      </c>
       <c r="D130" t="str">
         <v/>
       </c>
+      <c r="E130" t="str">
+        <v/>
+      </c>
     </row>
     <row r="131">
-      <c r="A131">
+      <c r="A131" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B131">
         <v>130</v>
       </c>
-      <c r="B131" t="str">
+      <c r="C131" t="str">
         <v>Open Walk/Trot HUS</v>
       </c>
-      <c r="C131" t="str">
-        <v/>
-      </c>
       <c r="D131" t="str">
         <v/>
       </c>
+      <c r="E131" t="str">
+        <v/>
+      </c>
     </row>
     <row r="132">
-      <c r="A132">
+      <c r="A132" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B132">
         <v>131</v>
       </c>
-      <c r="B132" t="str">
+      <c r="C132" t="str">
         <v>Junior Horse HUS</v>
       </c>
-      <c r="C132" t="str">
-        <v/>
-      </c>
       <c r="D132" t="str">
         <v/>
       </c>
+      <c r="E132" t="str">
+        <v/>
+      </c>
     </row>
     <row r="133">
-      <c r="A133">
+      <c r="A133" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B133">
         <v>132</v>
       </c>
-      <c r="B133" t="str">
+      <c r="C133" t="str">
         <v>Amateur HUS</v>
       </c>
-      <c r="C133" t="str">
-        <v/>
-      </c>
       <c r="D133" t="str">
         <v/>
       </c>
+      <c r="E133" t="str">
+        <v/>
+      </c>
     </row>
     <row r="134">
-      <c r="A134">
+      <c r="A134" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B134">
         <v>133</v>
       </c>
-      <c r="B134" t="str">
+      <c r="C134" t="str">
         <v>Select Amateur HUS</v>
       </c>
-      <c r="C134" t="str">
-        <v/>
-      </c>
       <c r="D134" t="str">
         <v/>
       </c>
+      <c r="E134" t="str">
+        <v/>
+      </c>
     </row>
     <row r="135">
-      <c r="A135">
+      <c r="A135" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B135">
         <v>134</v>
       </c>
-      <c r="B135" t="str">
+      <c r="C135" t="str">
         <v>Novice Amateur HUS</v>
       </c>
-      <c r="C135" t="str">
-        <v/>
-      </c>
       <c r="D135" t="str">
         <v/>
       </c>
+      <c r="E135" t="str">
+        <v/>
+      </c>
     </row>
     <row r="136">
-      <c r="A136">
+      <c r="A136" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B136">
         <v>135</v>
       </c>
-      <c r="B136" t="str">
+      <c r="C136" t="str">
         <v>Senior Horse HUS</v>
       </c>
-      <c r="C136" t="str">
-        <v/>
-      </c>
       <c r="D136" t="str">
         <v/>
       </c>
+      <c r="E136" t="str">
+        <v/>
+      </c>
     </row>
     <row r="137">
-      <c r="A137">
+      <c r="A137" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B137">
         <v>136</v>
       </c>
-      <c r="B137" t="str">
+      <c r="C137" t="str">
         <v>Beginner HUS</v>
       </c>
-      <c r="C137" t="str">
-        <v/>
-      </c>
       <c r="D137" t="str">
         <v/>
       </c>
+      <c r="E137" t="str">
+        <v/>
+      </c>
     </row>
     <row r="138">
-      <c r="A138">
+      <c r="A138" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B138">
         <v>137</v>
       </c>
-      <c r="B138" t="str">
+      <c r="C138" t="str">
         <v>Youth HUS 7-11 yrs</v>
       </c>
-      <c r="C138" t="str">
-        <v/>
-      </c>
       <c r="D138" t="str">
         <v/>
       </c>
+      <c r="E138" t="str">
+        <v/>
+      </c>
     </row>
     <row r="139">
-      <c r="A139">
+      <c r="A139" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B139">
         <v>138</v>
       </c>
-      <c r="B139" t="str">
+      <c r="C139" t="str">
         <v>Youth HUS 12-14 yrs</v>
       </c>
-      <c r="C139" t="str">
-        <v/>
-      </c>
       <c r="D139" t="str">
         <v/>
       </c>
+      <c r="E139" t="str">
+        <v/>
+      </c>
     </row>
     <row r="140">
-      <c r="A140">
+      <c r="A140" t="str">
+        <v>Hunter Under Saddle</v>
+      </c>
+      <c r="B140">
         <v>139</v>
       </c>
-      <c r="B140" t="str">
+      <c r="C140" t="str">
         <v>Youth HUS 15-18 yrs</v>
       </c>
-      <c r="C140" t="str">
-        <v/>
-      </c>
       <c r="D140" t="str">
         <v/>
       </c>
+      <c r="E140" t="str">
+        <v/>
+      </c>
     </row>
     <row r="141">
-      <c r="A141">
+      <c r="A141" t="str">
+        <v>Hunt Seat Equitation</v>
+      </c>
+      <c r="B141">
         <v>140</v>
       </c>
-      <c r="B141" t="str">
+      <c r="C141" t="str">
         <v>Amateur Hunt Seat Equitation</v>
       </c>
-      <c r="C141" t="str">
-        <v/>
-      </c>
       <c r="D141" t="str">
         <v/>
       </c>
+      <c r="E141" t="str">
+        <v/>
+      </c>
     </row>
     <row r="142">
-      <c r="A142">
+      <c r="A142" t="str">
+        <v>Hunt Seat Equitation</v>
+      </c>
+      <c r="B142">
         <v>141</v>
       </c>
-      <c r="B142" t="str">
+      <c r="C142" t="str">
         <v>Select Amateur Hunt Seat Equitation</v>
       </c>
-      <c r="C142" t="str">
-        <v/>
-      </c>
       <c r="D142" t="str">
         <v/>
       </c>
+      <c r="E142" t="str">
+        <v/>
+      </c>
     </row>
     <row r="143">
-      <c r="A143">
+      <c r="A143" t="str">
+        <v>Hunt Seat Equitation</v>
+      </c>
+      <c r="B143">
         <v>142</v>
       </c>
-      <c r="B143" t="str">
+      <c r="C143" t="str">
         <v>Novice Amateur Hunt Seat Equitation</v>
       </c>
-      <c r="C143" t="str">
-        <v/>
-      </c>
       <c r="D143" t="str">
         <v/>
       </c>
+      <c r="E143" t="str">
+        <v/>
+      </c>
     </row>
     <row r="144">
-      <c r="A144">
+      <c r="A144" t="str">
+        <v>Hunt Seat Equitation</v>
+      </c>
+      <c r="B144">
         <v>143</v>
       </c>
-      <c r="B144" t="str">
+      <c r="C144" t="str">
         <v>Beginner Hunt Seat Equitation</v>
       </c>
-      <c r="C144" t="str">
-        <v/>
-      </c>
       <c r="D144" t="str">
         <v/>
       </c>
+      <c r="E144" t="str">
+        <v/>
+      </c>
     </row>
     <row r="145">
-      <c r="A145">
+      <c r="A145" t="str">
+        <v>Hunt Seat Equitation</v>
+      </c>
+      <c r="B145">
         <v>144</v>
       </c>
-      <c r="B145" t="str">
+      <c r="C145" t="str">
         <v>Youth HSE 7-11 yrs</v>
       </c>
-      <c r="C145" t="str">
-        <v/>
-      </c>
       <c r="D145" t="str">
         <v/>
       </c>
+      <c r="E145" t="str">
+        <v/>
+      </c>
     </row>
     <row r="146">
-      <c r="A146">
+      <c r="A146" t="str">
+        <v>Hunt Seat Equitation</v>
+      </c>
+      <c r="B146">
         <v>145</v>
       </c>
-      <c r="B146" t="str">
+      <c r="C146" t="str">
         <v>Youth HSE 12-14 yrs</v>
       </c>
-      <c r="C146" t="str">
-        <v/>
-      </c>
       <c r="D146" t="str">
         <v/>
       </c>
+      <c r="E146" t="str">
+        <v/>
+      </c>
     </row>
     <row r="147">
-      <c r="A147">
+      <c r="A147" t="str">
+        <v>Hunt Seat Equitation</v>
+      </c>
+      <c r="B147">
         <v>146</v>
       </c>
-      <c r="B147" t="str">
+      <c r="C147" t="str">
         <v>Youth HSE 15-18 yrs</v>
       </c>
-      <c r="C147" t="str">
-        <v/>
-      </c>
       <c r="D147" t="str">
         <v/>
       </c>
+      <c r="E147" t="str">
+        <v/>
+      </c>
     </row>
     <row r="148">
-      <c r="A148">
+      <c r="A148" t="str">
+        <v>Hunt Seat Equitation</v>
+      </c>
+      <c r="B148">
         <v>147</v>
       </c>
-      <c r="B148" t="str">
+      <c r="C148" t="str">
         <v>EWD Hunt Seat Equitation</v>
       </c>
-      <c r="C148" t="str">
-        <v/>
-      </c>
       <c r="D148" t="str">
         <v/>
       </c>
+      <c r="E148" t="str">
+        <v/>
+      </c>
     </row>
     <row r="149">
-      <c r="A149">
+      <c r="A149" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B149">
         <v>148</v>
       </c>
-      <c r="B149" t="str">
+      <c r="C149" t="str">
         <v>1 yr old Led Trail</v>
       </c>
-      <c r="C149" t="str">
-        <v/>
-      </c>
       <c r="D149" t="str">
         <v/>
       </c>
+      <c r="E149" t="str">
+        <v/>
+      </c>
     </row>
     <row r="150">
-      <c r="A150">
+      <c r="A150" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B150">
         <v>149</v>
       </c>
-      <c r="B150" t="str">
+      <c r="C150" t="str">
         <v>2 yr old Led Trail</v>
       </c>
-      <c r="C150" t="str">
-        <v/>
-      </c>
       <c r="D150" t="str">
         <v/>
       </c>
+      <c r="E150" t="str">
+        <v/>
+      </c>
     </row>
     <row r="151">
-      <c r="A151">
+      <c r="A151" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B151">
         <v>150</v>
       </c>
-      <c r="B151" t="str">
+      <c r="C151" t="str">
         <v>3 yrs &amp; over Led Trail</v>
       </c>
-      <c r="C151" t="str">
-        <v/>
-      </c>
       <c r="D151" t="str">
         <v/>
       </c>
+      <c r="E151" t="str">
+        <v/>
+      </c>
     </row>
     <row r="152">
-      <c r="A152">
+      <c r="A152" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B152">
         <v>151</v>
       </c>
-      <c r="B152" t="str">
+      <c r="C152" t="str">
         <v>Open Walk/Jog Trail</v>
       </c>
-      <c r="C152" t="str">
-        <v/>
-      </c>
       <c r="D152" t="str">
         <v/>
       </c>
+      <c r="E152" t="str">
+        <v/>
+      </c>
     </row>
     <row r="153">
-      <c r="A153">
+      <c r="A153" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B153">
         <v>152</v>
       </c>
-      <c r="B153" t="str">
+      <c r="C153" t="str">
         <v>Junior Horse Trail</v>
       </c>
-      <c r="C153" t="str">
-        <v/>
-      </c>
       <c r="D153" t="str">
         <v/>
       </c>
+      <c r="E153" t="str">
+        <v/>
+      </c>
     </row>
     <row r="154">
-      <c r="A154">
+      <c r="A154" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B154">
         <v>153</v>
       </c>
-      <c r="B154" t="str">
+      <c r="C154" t="str">
         <v>Amateur Trail</v>
       </c>
-      <c r="C154" t="str">
-        <v/>
-      </c>
       <c r="D154" t="str">
         <v/>
       </c>
+      <c r="E154" t="str">
+        <v/>
+      </c>
     </row>
     <row r="155">
-      <c r="A155">
+      <c r="A155" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B155">
         <v>154</v>
       </c>
-      <c r="B155" t="str">
+      <c r="C155" t="str">
         <v>Select Amateur Trail</v>
       </c>
-      <c r="C155" t="str">
-        <v/>
-      </c>
       <c r="D155" t="str">
         <v/>
       </c>
+      <c r="E155" t="str">
+        <v/>
+      </c>
     </row>
     <row r="156">
-      <c r="A156">
+      <c r="A156" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B156">
         <v>155</v>
       </c>
-      <c r="B156" t="str">
+      <c r="C156" t="str">
         <v>Senior Horse Trail</v>
       </c>
-      <c r="C156" t="str">
-        <v/>
-      </c>
       <c r="D156" t="str">
         <v/>
       </c>
+      <c r="E156" t="str">
+        <v/>
+      </c>
     </row>
     <row r="157">
-      <c r="A157">
+      <c r="A157" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B157">
         <v>156</v>
       </c>
-      <c r="B157" t="str">
+      <c r="C157" t="str">
         <v>Novice Amateur Trail</v>
       </c>
-      <c r="C157" t="str">
-        <v/>
-      </c>
       <c r="D157" t="str">
         <v/>
       </c>
+      <c r="E157" t="str">
+        <v/>
+      </c>
     </row>
     <row r="158">
-      <c r="A158">
+      <c r="A158" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B158">
         <v>157</v>
       </c>
-      <c r="B158" t="str">
+      <c r="C158" t="str">
         <v>Beginner Trail</v>
       </c>
-      <c r="C158" t="str">
-        <v/>
-      </c>
       <c r="D158" t="str">
         <v/>
       </c>
+      <c r="E158" t="str">
+        <v/>
+      </c>
     </row>
     <row r="159">
-      <c r="A159">
+      <c r="A159" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B159">
         <v>158</v>
       </c>
-      <c r="B159" t="str">
+      <c r="C159" t="str">
         <v>Youth Trail 7-11 yrs</v>
       </c>
-      <c r="C159" t="str">
-        <v/>
-      </c>
       <c r="D159" t="str">
         <v/>
       </c>
+      <c r="E159" t="str">
+        <v/>
+      </c>
     </row>
     <row r="160">
-      <c r="A160">
+      <c r="A160" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B160">
         <v>159</v>
       </c>
-      <c r="B160" t="str">
+      <c r="C160" t="str">
         <v>Youth Trail 12-14 yrs</v>
       </c>
-      <c r="C160" t="str">
-        <v/>
-      </c>
       <c r="D160" t="str">
         <v/>
       </c>
+      <c r="E160" t="str">
+        <v/>
+      </c>
     </row>
     <row r="161">
-      <c r="A161">
+      <c r="A161" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B161">
         <v>160</v>
       </c>
-      <c r="B161" t="str">
+      <c r="C161" t="str">
         <v>Youth Trail 15-18 yrs</v>
       </c>
-      <c r="C161" t="str">
-        <v/>
-      </c>
       <c r="D161" t="str">
         <v/>
       </c>
+      <c r="E161" t="str">
+        <v/>
+      </c>
     </row>
     <row r="162">
-      <c r="A162">
+      <c r="A162" t="str">
+        <v>Trail</v>
+      </c>
+      <c r="B162">
         <v>161</v>
       </c>
-      <c r="B162" t="str">
+      <c r="C162" t="str">
         <v>EWD Trail</v>
       </c>
-      <c r="C162" t="str">
-        <v/>
-      </c>
       <c r="D162" t="str">
         <v/>
       </c>
+      <c r="E162" t="str">
+        <v/>
+      </c>
     </row>
     <row r="163">
-      <c r="A163">
+      <c r="A163" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B163">
         <v>162</v>
       </c>
-      <c r="B163" t="str">
+      <c r="C163" t="str">
         <v>Youth Lead Line 3-6 yrs</v>
       </c>
-      <c r="C163" t="str">
-        <v/>
-      </c>
       <c r="D163" t="str">
         <v/>
       </c>
+      <c r="E163" t="str">
+        <v/>
+      </c>
     </row>
     <row r="164">
-      <c r="A164">
+      <c r="A164" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B164">
         <v>163</v>
       </c>
-      <c r="B164" t="str">
+      <c r="C164" t="str">
         <v>Open Walk/Jog Western Pleasure</v>
       </c>
-      <c r="C164" t="str">
-        <v/>
-      </c>
       <c r="D164" t="str">
         <v/>
       </c>
+      <c r="E164" t="str">
+        <v/>
+      </c>
     </row>
     <row r="165">
-      <c r="A165">
+      <c r="A165" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B165">
         <v>164</v>
       </c>
-      <c r="B165" t="str">
+      <c r="C165" t="str">
         <v>Junior Horse Western Pleasure</v>
       </c>
-      <c r="C165" t="str">
-        <v/>
-      </c>
       <c r="D165" t="str">
         <v/>
       </c>
+      <c r="E165" t="str">
+        <v/>
+      </c>
     </row>
     <row r="166">
-      <c r="A166">
+      <c r="A166" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B166">
         <v>165</v>
       </c>
-      <c r="B166" t="str">
+      <c r="C166" t="str">
         <v>Amateur Western Pleasure</v>
       </c>
-      <c r="C166" t="str">
-        <v/>
-      </c>
       <c r="D166" t="str">
         <v/>
       </c>
+      <c r="E166" t="str">
+        <v/>
+      </c>
     </row>
     <row r="167">
-      <c r="A167">
+      <c r="A167" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B167">
         <v>166</v>
       </c>
-      <c r="B167" t="str">
+      <c r="C167" t="str">
         <v>Select Amateur Western Pleasure</v>
       </c>
-      <c r="C167" t="str">
-        <v/>
-      </c>
       <c r="D167" t="str">
         <v/>
       </c>
+      <c r="E167" t="str">
+        <v/>
+      </c>
     </row>
     <row r="168">
-      <c r="A168">
+      <c r="A168" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B168">
         <v>167</v>
       </c>
-      <c r="B168" t="str">
+      <c r="C168" t="str">
         <v>Novice Amateur Western Pleasure</v>
       </c>
-      <c r="C168" t="str">
-        <v/>
-      </c>
       <c r="D168" t="str">
         <v/>
       </c>
+      <c r="E168" t="str">
+        <v/>
+      </c>
     </row>
     <row r="169">
-      <c r="A169">
+      <c r="A169" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B169">
         <v>168</v>
       </c>
-      <c r="B169" t="str">
+      <c r="C169" t="str">
         <v>Senior Horse Western Pleasure</v>
       </c>
-      <c r="C169" t="str">
-        <v/>
-      </c>
       <c r="D169" t="str">
         <v/>
       </c>
+      <c r="E169" t="str">
+        <v/>
+      </c>
     </row>
     <row r="170">
-      <c r="A170">
+      <c r="A170" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B170">
         <v>169</v>
       </c>
-      <c r="B170" t="str">
+      <c r="C170" t="str">
         <v>Beginner Western Pleasure</v>
       </c>
-      <c r="C170" t="str">
-        <v/>
-      </c>
       <c r="D170" t="str">
         <v/>
       </c>
+      <c r="E170" t="str">
+        <v/>
+      </c>
     </row>
     <row r="171">
-      <c r="A171">
+      <c r="A171" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B171">
         <v>170</v>
       </c>
-      <c r="B171" t="str">
+      <c r="C171" t="str">
         <v>Youth WP 7-11 yrs</v>
       </c>
-      <c r="C171" t="str">
-        <v/>
-      </c>
       <c r="D171" t="str">
         <v/>
       </c>
+      <c r="E171" t="str">
+        <v/>
+      </c>
     </row>
     <row r="172">
-      <c r="A172">
+      <c r="A172" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B172">
         <v>171</v>
       </c>
-      <c r="B172" t="str">
+      <c r="C172" t="str">
         <v>Youth WP 12-14 yrs</v>
       </c>
-      <c r="C172" t="str">
-        <v/>
-      </c>
       <c r="D172" t="str">
         <v/>
       </c>
+      <c r="E172" t="str">
+        <v/>
+      </c>
     </row>
     <row r="173">
-      <c r="A173">
+      <c r="A173" t="str">
+        <v>Western Pleasure</v>
+      </c>
+      <c r="B173">
         <v>172</v>
       </c>
-      <c r="B173" t="str">
+      <c r="C173" t="str">
         <v>Youth WP 15-18 yrs</v>
       </c>
-      <c r="C173" t="str">
-        <v/>
-      </c>
       <c r="D173" t="str">
         <v/>
       </c>
+      <c r="E173" t="str">
+        <v/>
+      </c>
     </row>
     <row r="174">
-      <c r="A174">
+      <c r="A174" t="str">
+        <v>Horsemanship</v>
+      </c>
+      <c r="B174">
         <v>173</v>
       </c>
-      <c r="B174" t="str">
+      <c r="C174" t="str">
         <v>Open Horsemanship (HSAA Rules)</v>
       </c>
-      <c r="C174" t="str">
-        <v/>
-      </c>
       <c r="D174" t="str">
         <v/>
       </c>
+      <c r="E174" t="str">
+        <v/>
+      </c>
     </row>
     <row r="175">
-      <c r="A175">
+      <c r="A175" t="str">
+        <v>Horsemanship</v>
+      </c>
+      <c r="B175">
         <v>174</v>
       </c>
-      <c r="B175" t="str">
+      <c r="C175" t="str">
         <v>Amateur Horsemanship</v>
       </c>
-      <c r="C175" t="str">
-        <v/>
-      </c>
       <c r="D175" t="str">
         <v/>
       </c>
+      <c r="E175" t="str">
+        <v/>
+      </c>
     </row>
     <row r="176">
-      <c r="A176">
+      <c r="A176" t="str">
+        <v>Horsemanship</v>
+      </c>
+      <c r="B176">
         <v>175</v>
       </c>
-      <c r="B176" t="str">
+      <c r="C176" t="str">
         <v>Select Amateur Horsemanship</v>
       </c>
-      <c r="C176" t="str">
-        <v/>
-      </c>
       <c r="D176" t="str">
         <v/>
       </c>
+      <c r="E176" t="str">
+        <v/>
+      </c>
     </row>
     <row r="177">
-      <c r="A177">
+      <c r="A177" t="str">
+        <v>Horsemanship</v>
+      </c>
+      <c r="B177">
         <v>176</v>
       </c>
-      <c r="B177" t="str">
+      <c r="C177" t="str">
         <v>Novice Amateur Horsemanship</v>
       </c>
-      <c r="C177" t="str">
-        <v/>
-      </c>
       <c r="D177" t="str">
         <v/>
       </c>
+      <c r="E177" t="str">
+        <v/>
+      </c>
     </row>
     <row r="178">
-      <c r="A178">
+      <c r="A178" t="str">
+        <v>Horsemanship</v>
+      </c>
+      <c r="B178">
         <v>177</v>
       </c>
-      <c r="B178" t="str">
+      <c r="C178" t="str">
         <v>Beginner Horsemanship</v>
       </c>
-      <c r="C178" t="str">
-        <v/>
-      </c>
       <c r="D178" t="str">
         <v/>
       </c>
+      <c r="E178" t="str">
+        <v/>
+      </c>
     </row>
     <row r="179">
-      <c r="A179">
+      <c r="A179" t="str">
+        <v>Horsemanship</v>
+      </c>
+      <c r="B179">
         <v>178</v>
       </c>
-      <c r="B179" t="str">
+      <c r="C179" t="str">
         <v>Youth HMS 7-11 yrs</v>
       </c>
-      <c r="C179" t="str">
-        <v/>
-      </c>
       <c r="D179" t="str">
         <v/>
       </c>
+      <c r="E179" t="str">
+        <v/>
+      </c>
     </row>
     <row r="180">
-      <c r="A180">
+      <c r="A180" t="str">
+        <v>Horsemanship</v>
+      </c>
+      <c r="B180">
         <v>179</v>
       </c>
-      <c r="B180" t="str">
+      <c r="C180" t="str">
         <v>Youth HMS 12-14 yrs</v>
       </c>
-      <c r="C180" t="str">
-        <v/>
-      </c>
       <c r="D180" t="str">
         <v/>
       </c>
+      <c r="E180" t="str">
+        <v/>
+      </c>
     </row>
     <row r="181">
-      <c r="A181">
+      <c r="A181" t="str">
+        <v>Horsemanship</v>
+      </c>
+      <c r="B181">
         <v>180</v>
       </c>
-      <c r="B181" t="str">
+      <c r="C181" t="str">
         <v>Youth HMS 15-18 yrs</v>
       </c>
-      <c r="C181" t="str">
-        <v/>
-      </c>
       <c r="D181" t="str">
         <v/>
       </c>
+      <c r="E181" t="str">
+        <v/>
+      </c>
     </row>
     <row r="182">
-      <c r="A182">
+      <c r="A182" t="str">
+        <v>Horsemanship</v>
+      </c>
+      <c r="B182">
         <v>181</v>
       </c>
-      <c r="B182" t="str">
+      <c r="C182" t="str">
         <v>EWD Horsemanship</v>
       </c>
-      <c r="C182" t="str">
-        <v/>
-      </c>
       <c r="D182" t="str">
         <v/>
       </c>
+      <c r="E182" t="str">
+        <v/>
+      </c>
     </row>
     <row r="183">
-      <c r="A183">
+      <c r="A183" t="str">
+        <v>Ranch Riding</v>
+      </c>
+      <c r="B183">
         <v>182</v>
       </c>
-      <c r="B183" t="str">
+      <c r="C183" t="str">
         <v>Open Ranch Riding</v>
       </c>
-      <c r="C183" t="str">
-        <v/>
-      </c>
       <c r="D183" t="str">
         <v/>
       </c>
+      <c r="E183" t="str">
+        <v/>
+      </c>
     </row>
     <row r="184">
-      <c r="A184">
+      <c r="A184" t="str">
+        <v>Ranch Riding</v>
+      </c>
+      <c r="B184">
         <v>183</v>
       </c>
-      <c r="B184" t="str">
+      <c r="C184" t="str">
         <v>Amateur Ranch Riding</v>
       </c>
-      <c r="C184" t="str">
-        <v/>
-      </c>
       <c r="D184" t="str">
         <v/>
       </c>
+      <c r="E184" t="str">
+        <v/>
+      </c>
     </row>
     <row r="185">
-      <c r="A185">
+      <c r="A185" t="str">
+        <v>Ranch Riding</v>
+      </c>
+      <c r="B185">
         <v>184</v>
       </c>
-      <c r="B185" t="str">
+      <c r="C185" t="str">
         <v>Select Amateur Ranch Riding</v>
       </c>
-      <c r="C185" t="str">
-        <v/>
-      </c>
       <c r="D185" t="str">
         <v/>
       </c>
+      <c r="E185" t="str">
+        <v/>
+      </c>
     </row>
     <row r="186">
-      <c r="A186">
+      <c r="A186" t="str">
+        <v>Ranch Riding</v>
+      </c>
+      <c r="B186">
         <v>185</v>
       </c>
-      <c r="B186" t="str">
+      <c r="C186" t="str">
         <v>Novice Amateur Ranch Riding</v>
       </c>
-      <c r="C186" t="str">
-        <v/>
-      </c>
       <c r="D186" t="str">
         <v/>
       </c>
+      <c r="E186" t="str">
+        <v/>
+      </c>
     </row>
     <row r="187">
-      <c r="A187">
+      <c r="A187" t="str">
+        <v>Ranch Riding</v>
+      </c>
+      <c r="B187">
         <v>186</v>
       </c>
-      <c r="B187" t="str">
+      <c r="C187" t="str">
         <v>Beginner Ranch Riding</v>
       </c>
-      <c r="C187" t="str">
-        <v/>
-      </c>
       <c r="D187" t="str">
         <v/>
       </c>
+      <c r="E187" t="str">
+        <v/>
+      </c>
     </row>
     <row r="188">
-      <c r="A188">
+      <c r="A188" t="str">
+        <v>Ranch Riding</v>
+      </c>
+      <c r="B188">
         <v>187</v>
       </c>
-      <c r="B188" t="str">
+      <c r="C188" t="str">
         <v>Youth Ranch Riding 7-11 yrs</v>
       </c>
-      <c r="C188" t="str">
-        <v/>
-      </c>
       <c r="D188" t="str">
         <v/>
       </c>
+      <c r="E188" t="str">
+        <v/>
+      </c>
     </row>
     <row r="189">
-      <c r="A189">
+      <c r="A189" t="str">
+        <v>Ranch Riding</v>
+      </c>
+      <c r="B189">
         <v>188</v>
       </c>
-      <c r="B189" t="str">
+      <c r="C189" t="str">
         <v>Youth Ranch Riding 12-14 yrs</v>
       </c>
-      <c r="C189" t="str">
-        <v/>
-      </c>
       <c r="D189" t="str">
         <v/>
       </c>
+      <c r="E189" t="str">
+        <v/>
+      </c>
     </row>
     <row r="190">
-      <c r="A190">
+      <c r="A190" t="str">
+        <v>Ranch Riding</v>
+      </c>
+      <c r="B190">
         <v>189</v>
       </c>
-      <c r="B190" t="str">
+      <c r="C190" t="str">
         <v>Youth Ranch Riding 15-18 yrs</v>
       </c>
-      <c r="C190" t="str">
-        <v/>
-      </c>
       <c r="D190" t="str">
         <v/>
       </c>
+      <c r="E190" t="str">
+        <v/>
+      </c>
     </row>
     <row r="191">
-      <c r="A191">
+      <c r="A191" t="str">
+        <v>Reining</v>
+      </c>
+      <c r="B191">
         <v>190</v>
       </c>
-      <c r="B191" t="str">
+      <c r="C191" t="str">
         <v>Open Reining</v>
       </c>
-      <c r="C191" t="str">
-        <v/>
-      </c>
       <c r="D191" t="str">
         <v/>
       </c>
+      <c r="E191" t="str">
+        <v/>
+      </c>
     </row>
     <row r="192">
-      <c r="A192">
+      <c r="A192" t="str">
+        <v>Reining</v>
+      </c>
+      <c r="B192">
         <v>191</v>
       </c>
-      <c r="B192" t="str">
+      <c r="C192" t="str">
         <v>Amateur Reining</v>
       </c>
-      <c r="C192" t="str">
-        <v/>
-      </c>
       <c r="D192" t="str">
         <v/>
       </c>
+      <c r="E192" t="str">
+        <v/>
+      </c>
     </row>
     <row r="193">
-      <c r="A193">
+      <c r="A193" t="str">
+        <v>Reining</v>
+      </c>
+      <c r="B193">
         <v>192</v>
       </c>
-      <c r="B193" t="str">
+      <c r="C193" t="str">
         <v>Select Amateur Reining</v>
       </c>
-      <c r="C193" t="str">
-        <v/>
-      </c>
       <c r="D193" t="str">
         <v/>
       </c>
+      <c r="E193" t="str">
+        <v/>
+      </c>
     </row>
     <row r="194">
-      <c r="A194">
+      <c r="A194" t="str">
+        <v>Reining</v>
+      </c>
+      <c r="B194">
         <v>193</v>
       </c>
-      <c r="B194" t="str">
+      <c r="C194" t="str">
         <v>Novice Amateur Reining</v>
       </c>
-      <c r="C194" t="str">
-        <v/>
-      </c>
       <c r="D194" t="str">
         <v/>
       </c>
+      <c r="E194" t="str">
+        <v/>
+      </c>
     </row>
     <row r="195">
-      <c r="A195">
+      <c r="A195" t="str">
+        <v>Reining</v>
+      </c>
+      <c r="B195">
         <v>194</v>
       </c>
-      <c r="B195" t="str">
+      <c r="C195" t="str">
         <v>Youth Reining 7-11 yrs</v>
       </c>
-      <c r="C195" t="str">
-        <v/>
-      </c>
       <c r="D195" t="str">
         <v/>
       </c>
+      <c r="E195" t="str">
+        <v/>
+      </c>
     </row>
     <row r="196">
-      <c r="A196">
+      <c r="A196" t="str">
+        <v>Reining</v>
+      </c>
+      <c r="B196">
         <v>195</v>
       </c>
-      <c r="B196" t="str">
+      <c r="C196" t="str">
         <v>Youth Reining 12-14 yrs</v>
       </c>
-      <c r="C196" t="str">
-        <v/>
-      </c>
       <c r="D196" t="str">
         <v/>
       </c>
+      <c r="E196" t="str">
+        <v/>
+      </c>
     </row>
     <row r="197">
-      <c r="A197">
+      <c r="A197" t="str">
+        <v>Reining</v>
+      </c>
+      <c r="B197">
         <v>196</v>
       </c>
-      <c r="B197" t="str">
+      <c r="C197" t="str">
         <v>Youth Reining 15-18 yrs</v>
       </c>
-      <c r="C197" t="str">
-        <v/>
-      </c>
       <c r="D197" t="str">
+        <v/>
+      </c>
+      <c r="E197" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D197"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E197"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>